<commit_message>
feat(porth-integration): implement Kanban transitions based on Porth status - Added functionality to automatically transition Kanban statuses for purchase orders based on Porth updates. Configured stages for 'Consolidador', 'En tránsito', and 'Puerto' in the services configuration. This enhancement improves workflow automation and ensures accurate status representation in the Kanban board.
</commit_message>
<xml_diff>
--- a/Data viva/DATA VIVA_PRUEBAS.xlsx
+++ b/Data viva/DATA VIVA_PRUEBAS.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ocr0000143\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniel/Projects/Olo Orders/olo-raga-orders/Data viva/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45A6ADCD-0D31-3142-B758-4C158A1AA85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="15" windowWidth="13980" windowHeight="6795"/>
+    <workbookView xWindow="38040" yWindow="400" windowWidth="34200" windowHeight="21460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -17,14 +18,27 @@
     <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$BQ$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$BQ$18</definedName>
   </definedNames>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="750" uniqueCount="194">
   <si>
     <t>ORDER_NUMBER</t>
   </si>
@@ -236,9 +250,6 @@
     <t>Ingresada</t>
   </si>
   <si>
-    <t xml:space="preserve">WUHU XINGDIAN INDUSTRY CO., LTD                            </t>
-  </si>
-  <si>
     <t>Directo CR - FERRETERIA EPA, S.A.</t>
   </si>
   <si>
@@ -248,12 +259,6 @@
     <t>&lt;null&gt;</t>
   </si>
   <si>
-    <t>ASSHA510973</t>
-  </si>
-  <si>
-    <t>CAAU6958628</t>
-  </si>
-  <si>
     <t xml:space="preserve">FOB  </t>
   </si>
   <si>
@@ -264,15 +269,6 @@
   </si>
   <si>
     <t>-- N/A --</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CR #2 CNY Julio 25 </t>
-  </si>
-  <si>
-    <t>PICR6701044</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PICR6701044                   </t>
   </si>
   <si>
     <t>N</t>
@@ -629,7 +625,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -682,9 +678,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -722,9 +718,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -759,7 +755,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -794,7 +790,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -967,11 +963,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BQ19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:BQ18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1180,183 +1176,183 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>6701044</v>
+        <v>6701122</v>
       </c>
       <c r="B2" t="s">
         <v>69</v>
       </c>
       <c r="C2">
-        <v>327</v>
+        <v>865</v>
       </c>
       <c r="D2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E2">
+        <v>89</v>
+      </c>
+      <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="E2">
-        <v>85</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="G2" s="3">
+        <v>9028.5</v>
+      </c>
+      <c r="H2" t="s">
         <v>71</v>
       </c>
-      <c r="G2" s="1">
-        <v>37804</v>
-      </c>
-      <c r="H2" t="s">
-        <v>72</v>
-      </c>
       <c r="I2" s="2">
-        <v>45876</v>
+        <v>45877</v>
       </c>
       <c r="J2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K2">
         <v>2</v>
       </c>
       <c r="L2" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="M2">
         <v>23</v>
       </c>
       <c r="N2" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="O2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R2" s="2">
-        <v>45978</v>
+        <v>45965</v>
       </c>
       <c r="S2" s="2">
-        <v>45978</v>
+        <v>45965</v>
       </c>
       <c r="T2" s="2">
-        <v>45985</v>
+        <v>45945</v>
       </c>
       <c r="U2" s="2">
-        <v>45985</v>
+        <v>45971</v>
       </c>
       <c r="V2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W2">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="X2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y2" s="2">
-        <v>45998</v>
+        <v>45982</v>
       </c>
       <c r="Z2" s="2">
-        <v>46005</v>
+        <v>45991</v>
       </c>
       <c r="AA2" s="2">
-        <v>45998</v>
+        <v>45991</v>
       </c>
       <c r="AB2">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AC2" s="2">
-        <v>46045</v>
+        <v>46029</v>
       </c>
       <c r="AD2" s="2">
         <v>46060</v>
       </c>
       <c r="AE2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG2">
-        <v>7141</v>
+        <v>6946</v>
       </c>
       <c r="AH2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="AI2">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="AJ2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK2">
         <v>125</v>
       </c>
       <c r="AL2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="AM2" s="1">
-        <v>101346</v>
+        <v>101162</v>
       </c>
       <c r="AN2" s="2">
-        <v>46001</v>
+        <v>45982</v>
       </c>
       <c r="AO2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="AP2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AQ2" s="1">
-        <v>3320</v>
+        <v>4250</v>
       </c>
       <c r="AR2">
         <v>1000001</v>
       </c>
       <c r="AS2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT2" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="AU2" s="1">
-        <v>37804</v>
+        <v>9028</v>
       </c>
       <c r="AV2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="AW2" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX2" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="AY2" t="s">
         <v>77</v>
       </c>
       <c r="AZ2" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="BA2" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BB2" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE2" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="BF2">
         <v>2</v>
       </c>
-      <c r="BG2" t="s">
-        <v>73</v>
+      <c r="BG2" s="2">
+        <v>45848</v>
       </c>
       <c r="BH2">
         <v>14</v>
@@ -1365,207 +1361,204 @@
         <v>0</v>
       </c>
       <c r="BJ2" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ2" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="3" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>6701122</v>
+        <v>6701206</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="C3">
-        <v>865</v>
+        <v>462</v>
       </c>
       <c r="D3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E3">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="F3" t="s">
+        <v>91</v>
+      </c>
+      <c r="G3" s="3">
+        <v>22127.282999999999</v>
+      </c>
+      <c r="H3" t="s">
         <v>71</v>
       </c>
-      <c r="G3" s="3">
-        <v>9028.5</v>
-      </c>
-      <c r="H3" t="s">
-        <v>72</v>
-      </c>
       <c r="I3" s="2">
-        <v>45877</v>
+        <v>45883</v>
       </c>
       <c r="J3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K3">
         <v>2</v>
       </c>
       <c r="L3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="M3">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="O3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R3" s="2">
-        <v>45965</v>
+        <v>45982</v>
       </c>
       <c r="S3" s="2">
-        <v>45965</v>
+        <v>45986</v>
       </c>
       <c r="T3" s="2">
-        <v>45945</v>
+        <v>45922</v>
       </c>
       <c r="U3" s="2">
-        <v>45971</v>
+        <v>45989</v>
       </c>
       <c r="V3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W3">
-        <v>26</v>
+        <v>67</v>
       </c>
       <c r="X3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y3" s="2">
-        <v>45982</v>
+        <v>46001</v>
       </c>
       <c r="Z3" s="2">
-        <v>45991</v>
+        <v>46013</v>
       </c>
       <c r="AA3" s="2">
-        <v>45991</v>
+        <v>46001</v>
       </c>
       <c r="AB3">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AC3" s="2">
-        <v>46029</v>
+        <v>46052</v>
       </c>
       <c r="AD3" s="2">
-        <v>46060</v>
+        <v>46059</v>
       </c>
       <c r="AE3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG3">
-        <v>6946</v>
+        <v>7295</v>
       </c>
       <c r="AH3" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="AI3">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="AJ3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK3">
         <v>125</v>
       </c>
-      <c r="AL3" t="s">
-        <v>79</v>
-      </c>
-      <c r="AM3" s="1">
-        <v>101162</v>
-      </c>
-      <c r="AN3" s="2">
-        <v>45982</v>
+      <c r="AM3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>72</v>
       </c>
       <c r="AO3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="AP3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AQ3" s="1">
-        <v>4250</v>
+        <v>3320</v>
       </c>
       <c r="AR3">
         <v>1000001</v>
       </c>
       <c r="AS3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT3" t="s">
-        <v>92</v>
-      </c>
-      <c r="AU3" s="1">
-        <v>9028</v>
+        <v>96</v>
+      </c>
+      <c r="AU3" s="3">
+        <v>22127.279999999999</v>
       </c>
       <c r="AV3" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="AW3" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX3" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="AY3" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AZ3" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="BA3" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BB3" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE3" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="BF3">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="BG3" s="2">
-        <v>45848</v>
+        <v>45698</v>
       </c>
       <c r="BH3">
         <v>14</v>
@@ -1574,81 +1567,81 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ3" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="4" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>6701206</v>
+        <v>6701207</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C4">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="E4">
         <v>82</v>
       </c>
       <c r="F4" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="G4" s="3">
-        <v>22127.282999999999</v>
+        <v>11660.46</v>
       </c>
       <c r="H4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I4" s="2">
         <v>45883</v>
       </c>
       <c r="J4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K4">
         <v>2</v>
       </c>
       <c r="L4" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="M4">
         <v>22</v>
       </c>
       <c r="N4" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="O4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R4" s="2">
         <v>45982</v>
@@ -1663,13 +1656,13 @@
         <v>45989</v>
       </c>
       <c r="V4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W4">
         <v>67</v>
       </c>
       <c r="X4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y4" s="2">
         <v>46001</v>
@@ -1690,82 +1683,82 @@
         <v>46059</v>
       </c>
       <c r="AE4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG4">
         <v>7295</v>
       </c>
       <c r="AH4" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="AI4">
         <v>108</v>
       </c>
       <c r="AJ4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK4">
         <v>125</v>
       </c>
       <c r="AM4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AN4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AO4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="AP4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ4" s="1">
-        <v>3320</v>
+        <v>72</v>
+      </c>
+      <c r="AQ4" t="s">
+        <v>72</v>
       </c>
       <c r="AR4">
         <v>1000001</v>
       </c>
       <c r="AS4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT4" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="AU4" s="3">
-        <v>22127.279999999999</v>
+        <v>11660.46</v>
       </c>
       <c r="AV4" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="AW4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX4" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="AY4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AZ4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="BA4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BB4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE4" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="BF4">
         <v>8</v>
@@ -1780,204 +1773,207 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ4" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="5" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>6701207</v>
+        <v>6701296</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="C5">
-        <v>463</v>
+        <v>904</v>
       </c>
       <c r="D5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="E5">
         <v>82</v>
       </c>
       <c r="F5" t="s">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="G5" s="3">
-        <v>11660.46</v>
+        <v>26948.92</v>
       </c>
       <c r="H5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I5" s="2">
-        <v>45883</v>
+        <v>45890</v>
       </c>
       <c r="J5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K5">
         <v>2</v>
       </c>
       <c r="L5" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="M5">
         <v>22</v>
       </c>
       <c r="N5" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="O5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R5" s="2">
-        <v>45982</v>
+        <v>45968</v>
       </c>
       <c r="S5" s="2">
-        <v>45986</v>
+        <v>45968</v>
       </c>
       <c r="T5" s="2">
-        <v>45922</v>
+        <v>45937</v>
       </c>
       <c r="U5" s="2">
-        <v>45989</v>
+        <v>45991</v>
       </c>
       <c r="V5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W5">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="X5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y5" s="2">
-        <v>46001</v>
+        <v>45991</v>
       </c>
       <c r="Z5" s="2">
-        <v>46013</v>
+        <v>46005</v>
       </c>
       <c r="AA5" s="2">
-        <v>46001</v>
+        <v>45994</v>
       </c>
       <c r="AB5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AC5" s="2">
-        <v>46052</v>
+        <v>46037</v>
       </c>
       <c r="AD5" s="2">
-        <v>46059</v>
+        <v>46060</v>
       </c>
       <c r="AE5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG5">
-        <v>7295</v>
+        <v>7156</v>
       </c>
       <c r="AH5" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AI5">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="AJ5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK5">
         <v>125</v>
       </c>
-      <c r="AM5" t="s">
-        <v>73</v>
-      </c>
-      <c r="AN5" t="s">
-        <v>73</v>
+      <c r="AL5" t="s">
+        <v>76</v>
+      </c>
+      <c r="AM5" s="1">
+        <v>101367</v>
+      </c>
+      <c r="AN5" s="2">
+        <v>46003</v>
       </c>
       <c r="AO5" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="AP5" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ5" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="AQ5" s="1">
+        <v>4250</v>
       </c>
       <c r="AR5">
         <v>1000001</v>
       </c>
       <c r="AS5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT5" t="s">
         <v>105</v>
       </c>
       <c r="AU5" s="3">
-        <v>11660.46</v>
+        <v>26948.92</v>
       </c>
       <c r="AV5" t="s">
         <v>106</v>
       </c>
       <c r="AW5" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX5" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="AY5" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AZ5" t="s">
+        <v>72</v>
+      </c>
+      <c r="BA5" t="s">
+        <v>77</v>
+      </c>
+      <c r="BB5" t="s">
+        <v>77</v>
+      </c>
+      <c r="BC5" t="s">
+        <v>72</v>
+      </c>
+      <c r="BD5" t="s">
+        <v>72</v>
+      </c>
+      <c r="BE5" t="s">
         <v>107</v>
       </c>
-      <c r="BA5" t="s">
-        <v>83</v>
-      </c>
-      <c r="BB5" t="s">
-        <v>83</v>
-      </c>
-      <c r="BC5" t="s">
-        <v>73</v>
-      </c>
-      <c r="BD5" t="s">
-        <v>73</v>
-      </c>
-      <c r="BE5" t="s">
-        <v>85</v>
-      </c>
       <c r="BF5">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="BG5" s="2">
-        <v>45698</v>
+        <v>45848</v>
       </c>
       <c r="BH5">
         <v>14</v>
@@ -1986,33 +1982,33 @@
         <v>0</v>
       </c>
       <c r="BJ5" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ5" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="6" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>6701296</v>
+        <v>6701297</v>
       </c>
       <c r="B6" t="s">
         <v>69</v>
@@ -2021,46 +2017,46 @@
         <v>904</v>
       </c>
       <c r="D6" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="E6">
         <v>82</v>
       </c>
       <c r="F6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G6" s="3">
+        <v>26985.119999999999</v>
+      </c>
+      <c r="H6" t="s">
         <v>71</v>
-      </c>
-      <c r="G6" s="3">
-        <v>26948.92</v>
-      </c>
-      <c r="H6" t="s">
-        <v>72</v>
       </c>
       <c r="I6" s="2">
         <v>45890</v>
       </c>
       <c r="J6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K6">
         <v>2</v>
       </c>
       <c r="L6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="M6">
         <v>22</v>
       </c>
       <c r="N6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R6" s="2">
         <v>45968</v>
@@ -2072,16 +2068,16 @@
         <v>45937</v>
       </c>
       <c r="U6" s="2">
-        <v>45991</v>
+        <v>45989</v>
       </c>
       <c r="V6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W6">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="X6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y6" s="2">
         <v>45991</v>
@@ -2096,46 +2092,46 @@
         <v>3</v>
       </c>
       <c r="AC6" s="2">
-        <v>46037</v>
+        <v>46038</v>
       </c>
       <c r="AD6" s="2">
         <v>46060</v>
       </c>
       <c r="AE6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG6">
-        <v>7156</v>
+        <v>7150</v>
       </c>
       <c r="AH6" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="AI6">
         <v>91</v>
       </c>
       <c r="AJ6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK6">
         <v>125</v>
       </c>
       <c r="AL6" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="AM6" s="1">
-        <v>101367</v>
+        <v>101358</v>
       </c>
       <c r="AN6" s="2">
-        <v>46003</v>
+        <v>46002</v>
       </c>
       <c r="AO6" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="AP6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AQ6" s="1">
         <v>4250</v>
@@ -2144,43 +2140,43 @@
         <v>1000001</v>
       </c>
       <c r="AS6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT6" t="s">
+        <v>110</v>
+      </c>
+      <c r="AU6" s="3">
+        <v>26985.119999999999</v>
+      </c>
+      <c r="AV6" t="s">
         <v>111</v>
       </c>
-      <c r="AU6" s="3">
-        <v>26948.92</v>
-      </c>
-      <c r="AV6" t="s">
-        <v>112</v>
-      </c>
       <c r="AW6" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX6" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="AY6" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AZ6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BA6" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BB6" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE6" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="BF6">
         <v>2</v>
@@ -2195,201 +2191,201 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ6" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="7" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>6701297</v>
+        <v>6701353</v>
       </c>
       <c r="B7" t="s">
         <v>69</v>
       </c>
       <c r="C7">
-        <v>904</v>
+        <v>270</v>
       </c>
       <c r="D7" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E7">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F7" t="s">
+        <v>70</v>
+      </c>
+      <c r="G7" s="1">
+        <v>17712</v>
+      </c>
+      <c r="H7" t="s">
         <v>71</v>
       </c>
-      <c r="G7" s="3">
-        <v>26985.119999999999</v>
-      </c>
-      <c r="H7" t="s">
-        <v>72</v>
-      </c>
       <c r="I7" s="2">
-        <v>45890</v>
+        <v>45897</v>
       </c>
       <c r="J7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K7">
         <v>2</v>
       </c>
       <c r="L7" t="s">
+        <v>113</v>
+      </c>
+      <c r="M7">
+        <v>23</v>
+      </c>
+      <c r="N7" t="s">
         <v>114</v>
       </c>
-      <c r="M7">
-        <v>22</v>
-      </c>
-      <c r="N7" t="s">
-        <v>115</v>
-      </c>
       <c r="O7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R7" s="2">
-        <v>45968</v>
+        <v>45974</v>
       </c>
       <c r="S7" s="2">
-        <v>45968</v>
+        <v>45974</v>
       </c>
       <c r="T7" s="2">
-        <v>45937</v>
+        <v>45945</v>
       </c>
       <c r="U7" s="2">
-        <v>45989</v>
+        <v>45975</v>
       </c>
       <c r="V7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W7">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="X7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y7" s="2">
-        <v>45991</v>
+        <v>45984</v>
       </c>
       <c r="Z7" s="2">
-        <v>46005</v>
+        <v>46012</v>
       </c>
       <c r="AA7" s="2">
-        <v>45994</v>
+        <v>46004</v>
       </c>
       <c r="AB7">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="AC7" s="2">
-        <v>46038</v>
+        <v>46045</v>
       </c>
       <c r="AD7" s="2">
         <v>46060</v>
       </c>
       <c r="AE7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG7">
-        <v>7150</v>
+        <v>7207</v>
       </c>
       <c r="AH7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="AI7">
         <v>91</v>
       </c>
       <c r="AJ7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK7">
         <v>125</v>
       </c>
       <c r="AL7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="AM7" s="1">
-        <v>101358</v>
+        <v>101433</v>
       </c>
       <c r="AN7" s="2">
-        <v>46002</v>
+        <v>46009</v>
       </c>
       <c r="AO7" t="s">
-        <v>91</v>
+        <v>115</v>
       </c>
       <c r="AP7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AQ7" s="1">
-        <v>4250</v>
+        <v>3320</v>
       </c>
       <c r="AR7">
         <v>1000001</v>
       </c>
       <c r="AS7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT7" t="s">
         <v>116</v>
       </c>
-      <c r="AU7" s="3">
-        <v>26985.119999999999</v>
+      <c r="AU7" s="1">
+        <v>17712</v>
       </c>
       <c r="AV7" t="s">
         <v>117</v>
       </c>
       <c r="AW7" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX7" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="AY7" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="AZ7" t="s">
-        <v>73</v>
+        <v>118</v>
       </c>
       <c r="BA7" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BB7" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE7" t="s">
-        <v>113</v>
+        <v>79</v>
       </c>
       <c r="BF7">
         <v>2</v>
@@ -2404,207 +2400,207 @@
         <v>0</v>
       </c>
       <c r="BJ7" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ7" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="8" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>6701353</v>
+        <v>6701683</v>
       </c>
       <c r="B8" t="s">
         <v>69</v>
       </c>
       <c r="C8">
-        <v>270</v>
+        <v>380</v>
       </c>
       <c r="D8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E8">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F8" t="s">
+        <v>70</v>
+      </c>
+      <c r="G8" s="3">
+        <v>20570.05</v>
+      </c>
+      <c r="H8" t="s">
         <v>71</v>
       </c>
-      <c r="G8" s="1">
-        <v>17712</v>
-      </c>
-      <c r="H8" t="s">
-        <v>72</v>
-      </c>
       <c r="I8" s="2">
-        <v>45897</v>
+        <v>45911</v>
       </c>
       <c r="J8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K8">
         <v>2</v>
       </c>
       <c r="L8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="M8">
         <v>23</v>
       </c>
       <c r="N8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="O8" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P8" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q8" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R8" s="2">
-        <v>45974</v>
+        <v>45964</v>
       </c>
       <c r="S8" s="2">
-        <v>45974</v>
+        <v>45964</v>
       </c>
       <c r="T8" s="2">
-        <v>45945</v>
+        <v>45976</v>
       </c>
       <c r="U8" s="2">
-        <v>45975</v>
+        <v>45976</v>
       </c>
       <c r="V8" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W8">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="X8" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y8" s="2">
-        <v>45984</v>
+        <v>45983</v>
       </c>
       <c r="Z8" s="2">
-        <v>46012</v>
+        <v>46003</v>
       </c>
       <c r="AA8" s="2">
-        <v>46004</v>
+        <v>45991</v>
       </c>
       <c r="AB8">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="AC8" s="2">
-        <v>46045</v>
+        <v>46030</v>
       </c>
       <c r="AD8" s="2">
         <v>46060</v>
       </c>
       <c r="AE8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG8">
-        <v>7207</v>
+        <v>7130</v>
       </c>
       <c r="AH8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="AI8">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="AJ8" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK8">
         <v>125</v>
       </c>
       <c r="AL8" t="s">
+        <v>76</v>
+      </c>
+      <c r="AM8" s="1">
+        <v>101335</v>
+      </c>
+      <c r="AN8" s="2">
+        <v>46001</v>
+      </c>
+      <c r="AO8" t="s">
+        <v>122</v>
+      </c>
+      <c r="AP8" t="s">
+        <v>72</v>
+      </c>
+      <c r="AQ8" s="1">
+        <v>4290</v>
+      </c>
+      <c r="AR8">
+        <v>1000024</v>
+      </c>
+      <c r="AS8" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT8" t="s">
+        <v>123</v>
+      </c>
+      <c r="AU8" s="3">
+        <v>20570.05</v>
+      </c>
+      <c r="AV8" t="s">
+        <v>124</v>
+      </c>
+      <c r="AW8" t="s">
+        <v>77</v>
+      </c>
+      <c r="AX8" t="s">
+        <v>78</v>
+      </c>
+      <c r="AY8" t="s">
+        <v>74</v>
+      </c>
+      <c r="AZ8" t="s">
+        <v>125</v>
+      </c>
+      <c r="BA8" t="s">
+        <v>77</v>
+      </c>
+      <c r="BB8" t="s">
+        <v>77</v>
+      </c>
+      <c r="BC8" t="s">
+        <v>72</v>
+      </c>
+      <c r="BD8" t="s">
+        <v>72</v>
+      </c>
+      <c r="BE8" t="s">
         <v>79</v>
-      </c>
-      <c r="AM8" s="1">
-        <v>101433</v>
-      </c>
-      <c r="AN8" s="2">
-        <v>46009</v>
-      </c>
-      <c r="AO8" t="s">
-        <v>121</v>
-      </c>
-      <c r="AP8" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ8" s="1">
-        <v>3320</v>
-      </c>
-      <c r="AR8">
-        <v>1000001</v>
-      </c>
-      <c r="AS8" t="s">
-        <v>73</v>
-      </c>
-      <c r="AT8" t="s">
-        <v>122</v>
-      </c>
-      <c r="AU8" s="1">
-        <v>17712</v>
-      </c>
-      <c r="AV8" t="s">
-        <v>123</v>
-      </c>
-      <c r="AW8" t="s">
-        <v>83</v>
-      </c>
-      <c r="AX8" t="s">
-        <v>84</v>
-      </c>
-      <c r="AY8" t="s">
-        <v>77</v>
-      </c>
-      <c r="AZ8" t="s">
-        <v>124</v>
-      </c>
-      <c r="BA8" t="s">
-        <v>83</v>
-      </c>
-      <c r="BB8" t="s">
-        <v>83</v>
-      </c>
-      <c r="BC8" t="s">
-        <v>73</v>
-      </c>
-      <c r="BD8" t="s">
-        <v>73</v>
-      </c>
-      <c r="BE8" t="s">
-        <v>85</v>
       </c>
       <c r="BF8">
         <v>2</v>
       </c>
-      <c r="BG8" s="2">
-        <v>45848</v>
+      <c r="BG8" t="s">
+        <v>126</v>
       </c>
       <c r="BH8">
         <v>14</v>
@@ -2613,33 +2609,33 @@
         <v>0</v>
       </c>
       <c r="BJ8" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ8" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="9" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>6701683</v>
+        <v>6701684</v>
       </c>
       <c r="B9" t="s">
         <v>69</v>
@@ -2648,46 +2644,46 @@
         <v>380</v>
       </c>
       <c r="D9" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="E9">
         <v>85</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G9" s="3">
         <v>20570.05</v>
       </c>
       <c r="H9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I9" s="2">
         <v>45911</v>
       </c>
       <c r="J9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K9">
         <v>2</v>
       </c>
       <c r="L9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="M9">
         <v>23</v>
       </c>
       <c r="N9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="O9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R9" s="2">
         <v>45964</v>
@@ -2702,16 +2698,16 @@
         <v>45976</v>
       </c>
       <c r="V9" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W9">
         <v>0</v>
       </c>
       <c r="X9" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y9" s="2">
-        <v>45983</v>
+        <v>45982</v>
       </c>
       <c r="Z9" s="2">
         <v>46003</v>
@@ -2720,7 +2716,7 @@
         <v>45991</v>
       </c>
       <c r="AB9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AC9" s="2">
         <v>46030</v>
@@ -2729,91 +2725,91 @@
         <v>46060</v>
       </c>
       <c r="AE9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG9">
-        <v>7130</v>
+        <v>7132</v>
       </c>
       <c r="AH9" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="AI9">
         <v>77</v>
       </c>
       <c r="AJ9" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK9">
         <v>125</v>
       </c>
       <c r="AL9" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="AM9" s="1">
-        <v>101335</v>
+        <v>101337</v>
       </c>
       <c r="AN9" s="2">
         <v>46001</v>
       </c>
       <c r="AO9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AP9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AQ9" s="1">
-        <v>4290</v>
+        <v>4190</v>
       </c>
       <c r="AR9">
         <v>1000024</v>
       </c>
       <c r="AS9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="AU9" s="3">
         <v>20570.05</v>
       </c>
       <c r="AV9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AW9" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX9" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="AY9" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AZ9" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="BA9" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BB9" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE9" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="BF9">
         <v>2</v>
       </c>
       <c r="BG9" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="BH9">
         <v>14</v>
@@ -2822,207 +2818,204 @@
         <v>0</v>
       </c>
       <c r="BJ9" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ9" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="10" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>6701684</v>
+        <v>6701758</v>
       </c>
       <c r="B10" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="C10">
-        <v>380</v>
+        <v>903</v>
       </c>
       <c r="D10" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="E10">
         <v>85</v>
       </c>
       <c r="F10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G10" s="3">
+        <v>29145.119999999999</v>
+      </c>
+      <c r="H10" t="s">
         <v>71</v>
       </c>
-      <c r="G10" s="3">
-        <v>20570.05</v>
-      </c>
-      <c r="H10" t="s">
-        <v>72</v>
-      </c>
       <c r="I10" s="2">
-        <v>45911</v>
+        <v>45922</v>
       </c>
       <c r="J10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K10">
         <v>2</v>
       </c>
       <c r="L10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="M10">
         <v>23</v>
       </c>
       <c r="N10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R10" s="2">
-        <v>45964</v>
+        <v>45982</v>
       </c>
       <c r="S10" s="2">
-        <v>45964</v>
+        <v>45986</v>
       </c>
       <c r="T10" s="2">
-        <v>45976</v>
+        <v>45986</v>
       </c>
       <c r="U10" s="2">
-        <v>45976</v>
+        <v>45985</v>
       </c>
       <c r="V10" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W10">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="X10" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y10" s="2">
-        <v>45982</v>
+        <v>45991</v>
       </c>
       <c r="Z10" s="2">
-        <v>46003</v>
+        <v>45998</v>
       </c>
       <c r="AA10" s="2">
-        <v>45991</v>
+        <v>45992</v>
       </c>
       <c r="AB10">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AC10" s="2">
-        <v>46030</v>
+        <v>46029</v>
       </c>
       <c r="AD10" s="2">
         <v>46060</v>
       </c>
       <c r="AE10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG10">
-        <v>7132</v>
+        <v>7245</v>
       </c>
       <c r="AH10" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="AI10">
-        <v>77</v>
+        <v>36</v>
       </c>
       <c r="AJ10" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK10">
         <v>125</v>
       </c>
-      <c r="AL10" t="s">
+      <c r="AM10" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN10" t="s">
+        <v>72</v>
+      </c>
+      <c r="AO10" t="s">
+        <v>136</v>
+      </c>
+      <c r="AP10" t="s">
+        <v>72</v>
+      </c>
+      <c r="AQ10" s="1">
+        <v>4715</v>
+      </c>
+      <c r="AR10">
+        <v>1000001</v>
+      </c>
+      <c r="AS10" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT10" t="s">
+        <v>137</v>
+      </c>
+      <c r="AU10" s="3">
+        <v>29145.119999999999</v>
+      </c>
+      <c r="AV10" t="s">
+        <v>138</v>
+      </c>
+      <c r="AW10" t="s">
+        <v>77</v>
+      </c>
+      <c r="AX10" t="s">
+        <v>78</v>
+      </c>
+      <c r="AY10" t="s">
+        <v>77</v>
+      </c>
+      <c r="AZ10" t="s">
+        <v>139</v>
+      </c>
+      <c r="BA10" t="s">
+        <v>74</v>
+      </c>
+      <c r="BB10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BC10" t="s">
+        <v>72</v>
+      </c>
+      <c r="BD10" t="s">
+        <v>72</v>
+      </c>
+      <c r="BE10" t="s">
         <v>79</v>
-      </c>
-      <c r="AM10" s="1">
-        <v>101337</v>
-      </c>
-      <c r="AN10" s="2">
-        <v>46001</v>
-      </c>
-      <c r="AO10" t="s">
-        <v>135</v>
-      </c>
-      <c r="AP10" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ10" s="1">
-        <v>4190</v>
-      </c>
-      <c r="AR10">
-        <v>1000024</v>
-      </c>
-      <c r="AS10" t="s">
-        <v>73</v>
-      </c>
-      <c r="AT10" t="s">
-        <v>136</v>
-      </c>
-      <c r="AU10" s="3">
-        <v>20570.05</v>
-      </c>
-      <c r="AV10" t="s">
-        <v>137</v>
-      </c>
-      <c r="AW10" t="s">
-        <v>83</v>
-      </c>
-      <c r="AX10" t="s">
-        <v>84</v>
-      </c>
-      <c r="AY10" t="s">
-        <v>77</v>
-      </c>
-      <c r="AZ10" t="s">
-        <v>138</v>
-      </c>
-      <c r="BA10" t="s">
-        <v>83</v>
-      </c>
-      <c r="BB10" t="s">
-        <v>83</v>
-      </c>
-      <c r="BC10" t="s">
-        <v>73</v>
-      </c>
-      <c r="BD10" t="s">
-        <v>73</v>
-      </c>
-      <c r="BE10" t="s">
-        <v>85</v>
       </c>
       <c r="BF10">
         <v>2</v>
       </c>
-      <c r="BG10" t="s">
-        <v>132</v>
+      <c r="BG10" s="2">
+        <v>45972</v>
       </c>
       <c r="BH10">
         <v>14</v>
@@ -3031,204 +3024,207 @@
         <v>0</v>
       </c>
       <c r="BJ10" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ10" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="11" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A11">
-        <v>6701758</v>
+        <v>6701769</v>
       </c>
       <c r="B11" t="s">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="C11">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E11">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F11" t="s">
-        <v>97</v>
-      </c>
-      <c r="G11" s="3">
-        <v>29145.119999999999</v>
+        <v>70</v>
+      </c>
+      <c r="G11" s="1">
+        <v>13860</v>
       </c>
       <c r="H11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I11" s="2">
-        <v>45922</v>
+        <v>45923</v>
       </c>
       <c r="J11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K11">
         <v>2</v>
       </c>
       <c r="L11" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M11">
         <v>23</v>
       </c>
       <c r="N11" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R11" s="2">
-        <v>45982</v>
+        <v>45975</v>
       </c>
       <c r="S11" s="2">
+        <v>45975</v>
+      </c>
+      <c r="T11" s="2">
+        <v>45979</v>
+      </c>
+      <c r="U11" s="2">
         <v>45986</v>
       </c>
-      <c r="T11" s="2">
-        <v>45986</v>
-      </c>
-      <c r="U11" s="2">
-        <v>45985</v>
-      </c>
       <c r="V11" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="X11" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y11" s="2">
-        <v>45991</v>
+        <v>45994</v>
       </c>
       <c r="Z11" s="2">
-        <v>45998</v>
+        <v>46001</v>
       </c>
       <c r="AA11" s="2">
-        <v>45992</v>
+        <v>45994</v>
       </c>
       <c r="AB11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC11" s="2">
-        <v>46029</v>
+        <v>46038</v>
       </c>
       <c r="AD11" s="2">
         <v>46060</v>
       </c>
       <c r="AE11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG11">
-        <v>7245</v>
+        <v>7103</v>
       </c>
       <c r="AH11" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AI11">
-        <v>36</v>
+        <v>108</v>
       </c>
       <c r="AJ11" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK11">
         <v>125</v>
       </c>
-      <c r="AM11" t="s">
-        <v>73</v>
-      </c>
-      <c r="AN11" t="s">
-        <v>73</v>
+      <c r="AL11" t="s">
+        <v>76</v>
+      </c>
+      <c r="AM11" s="1">
+        <v>101298</v>
+      </c>
+      <c r="AN11" s="2">
+        <v>45999</v>
       </c>
       <c r="AO11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AP11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AQ11" s="1">
-        <v>4715</v>
+        <v>4250</v>
       </c>
       <c r="AR11">
         <v>1000001</v>
       </c>
       <c r="AS11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT11" t="s">
-        <v>143</v>
-      </c>
-      <c r="AU11" s="3">
-        <v>29145.119999999999</v>
+        <v>144</v>
+      </c>
+      <c r="AU11" s="1">
+        <v>13860</v>
       </c>
       <c r="AV11" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="AW11" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX11" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="AY11" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AZ11" t="s">
-        <v>145</v>
+        <v>72</v>
       </c>
       <c r="BA11" t="s">
         <v>77</v>
       </c>
       <c r="BB11" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE11" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="BF11">
         <v>2</v>
       </c>
-      <c r="BG11" s="2">
-        <v>45972</v>
+      <c r="BG11" t="s">
+        <v>147</v>
       </c>
       <c r="BH11">
         <v>14</v>
@@ -3237,81 +3233,81 @@
         <v>0</v>
       </c>
       <c r="BJ11" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ11" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="12" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>6701769</v>
+        <v>6701770</v>
       </c>
       <c r="B12" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="C12">
         <v>905</v>
       </c>
       <c r="D12" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E12">
         <v>89</v>
       </c>
       <c r="F12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G12" s="1">
+        <v>5841</v>
+      </c>
+      <c r="H12" t="s">
         <v>71</v>
-      </c>
-      <c r="G12" s="1">
-        <v>13860</v>
-      </c>
-      <c r="H12" t="s">
-        <v>72</v>
       </c>
       <c r="I12" s="2">
         <v>45923</v>
       </c>
       <c r="J12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K12">
         <v>2</v>
       </c>
       <c r="L12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="M12">
         <v>23</v>
       </c>
       <c r="N12" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="O12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R12" s="2">
         <v>45975</v>
@@ -3326,13 +3322,13 @@
         <v>45986</v>
       </c>
       <c r="V12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W12">
         <v>7</v>
       </c>
       <c r="X12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y12" s="2">
         <v>45994</v>
@@ -3353,91 +3349,88 @@
         <v>46060</v>
       </c>
       <c r="AE12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG12">
-        <v>7103</v>
+        <v>7190</v>
       </c>
       <c r="AH12" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="AI12">
         <v>108</v>
       </c>
       <c r="AJ12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK12">
         <v>125</v>
       </c>
-      <c r="AL12" t="s">
-        <v>79</v>
-      </c>
-      <c r="AM12" s="1">
-        <v>101298</v>
-      </c>
-      <c r="AN12" s="2">
-        <v>45999</v>
+      <c r="AM12" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN12" t="s">
+        <v>72</v>
       </c>
       <c r="AO12" t="s">
         <v>149</v>
       </c>
       <c r="AP12" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ12" s="1">
-        <v>4250</v>
+        <v>72</v>
+      </c>
+      <c r="AQ12" t="s">
+        <v>72</v>
       </c>
       <c r="AR12">
         <v>1000001</v>
       </c>
       <c r="AS12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT12" t="s">
         <v>150</v>
       </c>
       <c r="AU12" s="1">
-        <v>13860</v>
+        <v>5841</v>
       </c>
       <c r="AV12" t="s">
         <v>151</v>
       </c>
       <c r="AW12" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX12" t="s">
         <v>152</v>
       </c>
       <c r="AY12" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AZ12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BA12" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BB12" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE12" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="BF12">
         <v>2</v>
       </c>
       <c r="BG12" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="BH12">
         <v>14</v>
@@ -3446,81 +3439,81 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ12" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="13" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A13">
-        <v>6701770</v>
+        <v>6701771</v>
       </c>
       <c r="B13" t="s">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="C13">
         <v>905</v>
       </c>
       <c r="D13" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E13">
         <v>89</v>
       </c>
       <c r="F13" t="s">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="G13" s="1">
-        <v>5841</v>
+        <v>2720</v>
       </c>
       <c r="H13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I13" s="2">
         <v>45923</v>
       </c>
       <c r="J13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K13">
         <v>2</v>
       </c>
       <c r="L13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="M13">
         <v>23</v>
       </c>
       <c r="N13" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="O13" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P13" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q13" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R13" s="2">
         <v>45975</v>
@@ -3535,13 +3528,13 @@
         <v>45986</v>
       </c>
       <c r="V13" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W13">
         <v>7</v>
       </c>
       <c r="X13" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y13" s="2">
         <v>45994</v>
@@ -3550,100 +3543,103 @@
         <v>46001</v>
       </c>
       <c r="AA13" s="2">
-        <v>45994</v>
+        <v>45997</v>
       </c>
       <c r="AB13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AC13" s="2">
-        <v>46038</v>
+        <v>46037</v>
       </c>
       <c r="AD13" s="2">
         <v>46060</v>
       </c>
       <c r="AE13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG13">
-        <v>7190</v>
+        <v>7104</v>
       </c>
       <c r="AH13" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AI13">
         <v>108</v>
       </c>
       <c r="AJ13" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK13">
         <v>125</v>
       </c>
-      <c r="AM13" t="s">
-        <v>73</v>
-      </c>
-      <c r="AN13" t="s">
-        <v>73</v>
+      <c r="AL13" t="s">
+        <v>76</v>
+      </c>
+      <c r="AM13" s="1">
+        <v>101299</v>
+      </c>
+      <c r="AN13" s="2">
+        <v>45999</v>
       </c>
       <c r="AO13" t="s">
         <v>155</v>
       </c>
       <c r="AP13" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ13" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="AQ13" s="1">
+        <v>3320</v>
       </c>
       <c r="AR13">
         <v>1000001</v>
       </c>
       <c r="AS13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT13" t="s">
         <v>156</v>
       </c>
       <c r="AU13" s="1">
-        <v>5841</v>
+        <v>2720</v>
       </c>
       <c r="AV13" t="s">
         <v>157</v>
       </c>
       <c r="AW13" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX13" t="s">
         <v>158</v>
       </c>
       <c r="AY13" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AZ13" t="s">
-        <v>73</v>
+        <v>159</v>
       </c>
       <c r="BA13" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BB13" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE13" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="BF13">
         <v>2</v>
       </c>
       <c r="BG13" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="BH13">
         <v>14</v>
@@ -3652,81 +3648,81 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ13" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="14" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>6701771</v>
+        <v>6701772</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="C14">
         <v>905</v>
       </c>
       <c r="D14" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E14">
         <v>89</v>
       </c>
       <c r="F14" t="s">
+        <v>91</v>
+      </c>
+      <c r="G14" s="1">
+        <v>18305</v>
+      </c>
+      <c r="H14" t="s">
         <v>71</v>
-      </c>
-      <c r="G14" s="1">
-        <v>2720</v>
-      </c>
-      <c r="H14" t="s">
-        <v>72</v>
       </c>
       <c r="I14" s="2">
         <v>45923</v>
       </c>
       <c r="J14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K14">
         <v>2</v>
       </c>
       <c r="L14" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="M14">
         <v>23</v>
       </c>
       <c r="N14" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="O14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R14" s="2">
         <v>45975</v>
@@ -3738,22 +3734,22 @@
         <v>45979</v>
       </c>
       <c r="U14" s="2">
-        <v>45986</v>
+        <v>45985</v>
       </c>
       <c r="V14" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W14">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X14" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y14" s="2">
         <v>45994</v>
       </c>
       <c r="Z14" s="2">
-        <v>46001</v>
+        <v>46008</v>
       </c>
       <c r="AA14" s="2">
         <v>45997</v>
@@ -3768,91 +3764,88 @@
         <v>46060</v>
       </c>
       <c r="AE14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG14">
-        <v>7104</v>
+        <v>7227</v>
       </c>
       <c r="AH14" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="AI14">
         <v>108</v>
       </c>
       <c r="AJ14" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK14">
         <v>125</v>
       </c>
-      <c r="AL14" t="s">
-        <v>79</v>
-      </c>
-      <c r="AM14" s="1">
-        <v>101299</v>
-      </c>
-      <c r="AN14" s="2">
-        <v>45999</v>
+      <c r="AM14" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN14" t="s">
+        <v>72</v>
       </c>
       <c r="AO14" t="s">
         <v>161</v>
       </c>
       <c r="AP14" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ14" s="1">
-        <v>3320</v>
+        <v>72</v>
+      </c>
+      <c r="AQ14" t="s">
+        <v>72</v>
       </c>
       <c r="AR14">
         <v>1000001</v>
       </c>
       <c r="AS14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT14" t="s">
         <v>162</v>
       </c>
       <c r="AU14" s="1">
-        <v>2720</v>
+        <v>18305</v>
       </c>
       <c r="AV14" t="s">
         <v>163</v>
       </c>
       <c r="AW14" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX14" t="s">
         <v>164</v>
       </c>
       <c r="AY14" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AZ14" t="s">
-        <v>165</v>
+        <v>72</v>
       </c>
       <c r="BA14" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BB14" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE14" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="BF14">
         <v>2</v>
       </c>
       <c r="BG14" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="BH14">
         <v>14</v>
@@ -3861,60 +3854,60 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ14" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="15" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A15">
-        <v>6701772</v>
+        <v>6702103</v>
       </c>
       <c r="B15" t="s">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="C15">
-        <v>905</v>
+        <v>913</v>
       </c>
       <c r="D15" t="s">
-        <v>146</v>
+        <v>165</v>
       </c>
       <c r="E15">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F15" t="s">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="G15" s="1">
-        <v>18305</v>
+        <v>13090</v>
       </c>
       <c r="H15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I15" s="2">
-        <v>45923</v>
+        <v>45951</v>
       </c>
       <c r="J15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K15">
         <v>2</v>
@@ -3926,222 +3919,225 @@
         <v>23</v>
       </c>
       <c r="N15" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="O15" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P15" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q15" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R15" s="2">
-        <v>45975</v>
+        <v>45994</v>
       </c>
       <c r="S15" s="2">
-        <v>45975</v>
+        <v>45994</v>
       </c>
       <c r="T15" s="2">
-        <v>45979</v>
+        <v>45999</v>
       </c>
       <c r="U15" s="2">
-        <v>45985</v>
+        <v>45991</v>
       </c>
       <c r="V15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W15">
-        <v>6</v>
+        <v>-8</v>
       </c>
       <c r="X15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y15" s="2">
-        <v>45994</v>
+        <v>46003</v>
       </c>
       <c r="Z15" s="2">
-        <v>46008</v>
+        <v>46010</v>
       </c>
       <c r="AA15" s="2">
-        <v>45997</v>
+        <v>46003</v>
       </c>
       <c r="AB15">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AC15" s="2">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="AD15" s="2">
         <v>46060</v>
       </c>
       <c r="AE15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG15">
-        <v>7227</v>
+        <v>7192</v>
       </c>
       <c r="AH15" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AI15">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="AJ15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK15">
         <v>125</v>
       </c>
-      <c r="AM15" t="s">
-        <v>73</v>
-      </c>
-      <c r="AN15" t="s">
-        <v>73</v>
+      <c r="AL15" t="s">
+        <v>76</v>
+      </c>
+      <c r="AM15" s="1">
+        <v>101418</v>
+      </c>
+      <c r="AN15" s="2">
+        <v>46008</v>
       </c>
       <c r="AO15" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AP15" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ15" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="AQ15" s="1">
+        <v>3125</v>
       </c>
       <c r="AR15">
-        <v>1000001</v>
+        <v>1000007</v>
       </c>
       <c r="AS15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="AU15" s="1">
-        <v>18305</v>
+        <v>13090</v>
       </c>
       <c r="AV15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="AW15" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX15" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AY15" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AZ15" t="s">
-        <v>73</v>
+        <v>172</v>
       </c>
       <c r="BA15" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BB15" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE15" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="BF15">
         <v>2</v>
       </c>
-      <c r="BG15" t="s">
-        <v>153</v>
+      <c r="BG15" s="2">
+        <v>45700</v>
       </c>
       <c r="BH15">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="BI15">
         <v>0</v>
       </c>
       <c r="BJ15" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ15" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="16" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A16">
-        <v>6702103</v>
+        <v>6702104</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="C16">
         <v>913</v>
       </c>
       <c r="D16" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="E16">
         <v>85</v>
       </c>
       <c r="F16" t="s">
+        <v>91</v>
+      </c>
+      <c r="G16" s="1">
+        <v>5950</v>
+      </c>
+      <c r="H16" t="s">
         <v>71</v>
-      </c>
-      <c r="G16" s="1">
-        <v>13090</v>
-      </c>
-      <c r="H16" t="s">
-        <v>72</v>
       </c>
       <c r="I16" s="2">
         <v>45951</v>
       </c>
       <c r="J16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K16">
         <v>2</v>
       </c>
       <c r="L16" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="M16">
         <v>23</v>
       </c>
       <c r="N16" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="O16" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P16" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q16" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R16" s="2">
         <v>45994</v>
@@ -4156,19 +4152,19 @@
         <v>45991</v>
       </c>
       <c r="V16" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W16">
         <v>-8</v>
       </c>
       <c r="X16" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y16" s="2">
         <v>46003</v>
       </c>
       <c r="Z16" s="2">
-        <v>46010</v>
+        <v>46017</v>
       </c>
       <c r="AA16" s="2">
         <v>46003</v>
@@ -4183,85 +4179,82 @@
         <v>46060</v>
       </c>
       <c r="AE16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG16">
-        <v>7192</v>
+        <v>7461</v>
       </c>
       <c r="AH16" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="AI16">
         <v>92</v>
       </c>
       <c r="AJ16" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK16">
         <v>125</v>
       </c>
-      <c r="AL16" t="s">
-        <v>79</v>
-      </c>
-      <c r="AM16" s="1">
-        <v>101418</v>
-      </c>
-      <c r="AN16" s="2">
-        <v>46008</v>
+      <c r="AM16" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN16" t="s">
+        <v>72</v>
       </c>
       <c r="AO16" t="s">
         <v>174</v>
       </c>
       <c r="AP16" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ16" s="1">
-        <v>3125</v>
+        <v>72</v>
+      </c>
+      <c r="AQ16" t="s">
+        <v>72</v>
       </c>
       <c r="AR16">
         <v>1000007</v>
       </c>
       <c r="AS16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT16" t="s">
         <v>175</v>
       </c>
       <c r="AU16" s="1">
-        <v>13090</v>
+        <v>5950</v>
       </c>
       <c r="AV16" t="s">
         <v>176</v>
       </c>
       <c r="AW16" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX16" t="s">
         <v>177</v>
       </c>
       <c r="AY16" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AZ16" t="s">
         <v>178</v>
       </c>
       <c r="BA16" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BB16" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE16" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="BF16">
         <v>2</v>
@@ -4276,266 +4269,269 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ16" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="17" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A17">
-        <v>6702104</v>
+        <v>6702106</v>
       </c>
       <c r="B17" t="s">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="C17">
-        <v>913</v>
+        <v>494</v>
       </c>
       <c r="D17" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="E17">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F17" t="s">
-        <v>97</v>
-      </c>
-      <c r="G17" s="1">
-        <v>5950</v>
+        <v>70</v>
+      </c>
+      <c r="G17" s="3">
+        <v>22673.74</v>
       </c>
       <c r="H17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I17" s="2">
         <v>45951</v>
       </c>
       <c r="J17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K17">
         <v>2</v>
       </c>
       <c r="L17" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="M17">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="N17" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="O17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R17" s="2">
-        <v>45994</v>
+        <v>45979</v>
       </c>
       <c r="S17" s="2">
-        <v>45994</v>
+        <v>45979</v>
       </c>
       <c r="T17" s="2">
-        <v>45999</v>
+        <v>46001</v>
       </c>
       <c r="U17" s="2">
-        <v>45991</v>
+        <v>45983</v>
       </c>
       <c r="V17" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W17">
-        <v>-8</v>
+        <v>-18</v>
       </c>
       <c r="X17" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y17" s="2">
-        <v>46003</v>
+        <v>46001</v>
       </c>
       <c r="Z17" s="2">
-        <v>46017</v>
+        <v>46034</v>
       </c>
       <c r="AA17" s="2">
-        <v>46003</v>
+        <v>46009</v>
       </c>
       <c r="AB17">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AC17" s="2">
-        <v>46045</v>
+        <v>46052</v>
       </c>
       <c r="AD17" s="2">
-        <v>46060</v>
+        <v>46059</v>
       </c>
       <c r="AE17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG17">
-        <v>7461</v>
+        <v>7510</v>
       </c>
       <c r="AH17" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AI17">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="AJ17" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK17">
         <v>125</v>
       </c>
-      <c r="AM17" t="s">
-        <v>73</v>
-      </c>
-      <c r="AN17" t="s">
-        <v>73</v>
+      <c r="AL17" t="s">
+        <v>76</v>
+      </c>
+      <c r="AM17" s="1">
+        <v>101761</v>
+      </c>
+      <c r="AN17" s="2">
+        <v>46055</v>
       </c>
       <c r="AO17" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="AP17" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ17" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="AQ17" s="1">
+        <v>3320</v>
       </c>
       <c r="AR17">
-        <v>1000007</v>
+        <v>1000001</v>
       </c>
       <c r="AS17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT17" t="s">
-        <v>181</v>
-      </c>
-      <c r="AU17" s="1">
-        <v>5950</v>
+        <v>183</v>
+      </c>
+      <c r="AU17" s="3">
+        <v>22673.74</v>
       </c>
       <c r="AV17" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="AW17" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AX17" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="AY17" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="AZ17" t="s">
-        <v>184</v>
+        <v>72</v>
       </c>
       <c r="BA17" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BB17" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE17" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="BF17">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="BG17" s="2">
-        <v>45700</v>
+        <v>45819</v>
       </c>
       <c r="BH17">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="BI17">
         <v>0</v>
       </c>
       <c r="BJ17" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ17" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="18" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A18">
-        <v>6702106</v>
+        <v>6702107</v>
       </c>
       <c r="B18" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="C18">
         <v>494</v>
       </c>
       <c r="D18" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="E18">
         <v>83</v>
       </c>
       <c r="F18" t="s">
+        <v>91</v>
+      </c>
+      <c r="G18" s="3">
+        <v>58880.98</v>
+      </c>
+      <c r="H18" t="s">
         <v>71</v>
-      </c>
-      <c r="G18" s="3">
-        <v>22673.74</v>
-      </c>
-      <c r="H18" t="s">
-        <v>72</v>
       </c>
       <c r="I18" s="2">
         <v>45951</v>
       </c>
       <c r="J18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K18">
         <v>2</v>
@@ -4544,19 +4540,19 @@
         <v>186</v>
       </c>
       <c r="M18">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="N18" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="O18" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P18" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q18" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R18" s="2">
         <v>45979</v>
@@ -4571,13 +4567,13 @@
         <v>45983</v>
       </c>
       <c r="V18" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W18">
         <v>-18</v>
       </c>
       <c r="X18" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Y18" s="2">
         <v>46001</v>
@@ -4598,85 +4594,82 @@
         <v>46059</v>
       </c>
       <c r="AE18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AG18">
-        <v>7510</v>
+        <v>7474</v>
       </c>
       <c r="AH18" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="AI18">
         <v>71</v>
       </c>
       <c r="AJ18" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK18">
         <v>125</v>
       </c>
-      <c r="AL18" t="s">
-        <v>79</v>
-      </c>
-      <c r="AM18" s="1">
-        <v>101761</v>
-      </c>
-      <c r="AN18" s="2">
-        <v>46055</v>
+      <c r="AM18" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN18" t="s">
+        <v>72</v>
       </c>
       <c r="AO18" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AP18" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ18" s="1">
-        <v>3320</v>
+        <v>72</v>
+      </c>
+      <c r="AQ18" t="s">
+        <v>72</v>
       </c>
       <c r="AR18">
         <v>1000001</v>
       </c>
       <c r="AS18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AT18" t="s">
+        <v>188</v>
+      </c>
+      <c r="AU18" s="3">
+        <v>58880.98</v>
+      </c>
+      <c r="AV18" t="s">
         <v>189</v>
       </c>
-      <c r="AU18" s="3">
-        <v>22673.74</v>
-      </c>
-      <c r="AV18" t="s">
+      <c r="AW18" t="s">
+        <v>77</v>
+      </c>
+      <c r="AX18" t="s">
         <v>190</v>
       </c>
-      <c r="AW18" t="s">
-        <v>83</v>
-      </c>
-      <c r="AX18" t="s">
+      <c r="AY18" t="s">
+        <v>77</v>
+      </c>
+      <c r="AZ18" t="s">
         <v>191</v>
       </c>
-      <c r="AY18" t="s">
-        <v>77</v>
-      </c>
-      <c r="AZ18" t="s">
-        <v>73</v>
-      </c>
       <c r="BA18" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BB18" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="BC18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BD18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BE18" t="s">
-        <v>85</v>
+        <v>192</v>
       </c>
       <c r="BF18">
         <v>8</v>
@@ -4691,255 +4684,49 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="BK18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BL18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BM18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BN18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BO18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BP18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="BQ18" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="19" spans="1:69" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>6702107</v>
-      </c>
-      <c r="B19" t="s">
-        <v>95</v>
-      </c>
-      <c r="C19">
-        <v>494</v>
-      </c>
-      <c r="D19" t="s">
-        <v>185</v>
-      </c>
-      <c r="E19">
-        <v>83</v>
-      </c>
-      <c r="F19" t="s">
-        <v>97</v>
-      </c>
-      <c r="G19" s="3">
-        <v>58880.98</v>
-      </c>
-      <c r="H19" t="s">
-        <v>72</v>
-      </c>
-      <c r="I19" s="2">
-        <v>45951</v>
-      </c>
-      <c r="J19" t="s">
-        <v>73</v>
-      </c>
-      <c r="K19">
-        <v>2</v>
-      </c>
-      <c r="L19" t="s">
-        <v>192</v>
-      </c>
-      <c r="M19">
-        <v>25</v>
-      </c>
-      <c r="N19" t="s">
-        <v>187</v>
-      </c>
-      <c r="O19" t="s">
-        <v>76</v>
-      </c>
-      <c r="P19" t="s">
-        <v>76</v>
-      </c>
-      <c r="Q19" t="s">
-        <v>76</v>
-      </c>
-      <c r="R19" s="2">
-        <v>45979</v>
-      </c>
-      <c r="S19" s="2">
-        <v>45979</v>
-      </c>
-      <c r="T19" s="2">
-        <v>46001</v>
-      </c>
-      <c r="U19" s="2">
-        <v>45983</v>
-      </c>
-      <c r="V19" t="s">
-        <v>77</v>
-      </c>
-      <c r="W19">
-        <v>-18</v>
-      </c>
-      <c r="X19" t="s">
-        <v>77</v>
-      </c>
-      <c r="Y19" s="2">
-        <v>46001</v>
-      </c>
-      <c r="Z19" s="2">
-        <v>46034</v>
-      </c>
-      <c r="AA19" s="2">
-        <v>46009</v>
-      </c>
-      <c r="AB19">
-        <v>8</v>
-      </c>
-      <c r="AC19" s="2">
-        <v>46052</v>
-      </c>
-      <c r="AD19" s="2">
-        <v>46059</v>
-      </c>
-      <c r="AE19" t="s">
-        <v>73</v>
-      </c>
-      <c r="AF19" t="s">
-        <v>73</v>
-      </c>
-      <c r="AG19">
-        <v>7474</v>
-      </c>
-      <c r="AH19" t="s">
-        <v>100</v>
-      </c>
-      <c r="AI19">
-        <v>71</v>
-      </c>
-      <c r="AJ19" t="s">
-        <v>77</v>
-      </c>
-      <c r="AK19">
-        <v>125</v>
-      </c>
-      <c r="AM19" t="s">
-        <v>73</v>
-      </c>
-      <c r="AN19" t="s">
-        <v>73</v>
-      </c>
-      <c r="AO19" t="s">
         <v>193</v>
-      </c>
-      <c r="AP19" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ19" t="s">
-        <v>73</v>
-      </c>
-      <c r="AR19">
-        <v>1000001</v>
-      </c>
-      <c r="AS19" t="s">
-        <v>73</v>
-      </c>
-      <c r="AT19" t="s">
-        <v>194</v>
-      </c>
-      <c r="AU19" s="3">
-        <v>58880.98</v>
-      </c>
-      <c r="AV19" t="s">
-        <v>195</v>
-      </c>
-      <c r="AW19" t="s">
-        <v>83</v>
-      </c>
-      <c r="AX19" t="s">
-        <v>196</v>
-      </c>
-      <c r="AY19" t="s">
-        <v>83</v>
-      </c>
-      <c r="AZ19" t="s">
-        <v>197</v>
-      </c>
-      <c r="BA19" t="s">
-        <v>83</v>
-      </c>
-      <c r="BB19" t="s">
-        <v>83</v>
-      </c>
-      <c r="BC19" t="s">
-        <v>73</v>
-      </c>
-      <c r="BD19" t="s">
-        <v>73</v>
-      </c>
-      <c r="BE19" t="s">
-        <v>198</v>
-      </c>
-      <c r="BF19">
-        <v>8</v>
-      </c>
-      <c r="BG19" s="2">
-        <v>45819</v>
-      </c>
-      <c r="BH19">
-        <v>14</v>
-      </c>
-      <c r="BI19">
-        <v>0</v>
-      </c>
-      <c r="BJ19" t="s">
-        <v>86</v>
-      </c>
-      <c r="BK19" t="s">
-        <v>73</v>
-      </c>
-      <c r="BL19" t="s">
-        <v>73</v>
-      </c>
-      <c r="BM19" t="s">
-        <v>73</v>
-      </c>
-      <c r="BN19" t="s">
-        <v>73</v>
-      </c>
-      <c r="BO19" t="s">
-        <v>73</v>
-      </c>
-      <c r="BP19" t="s">
-        <v>73</v>
-      </c>
-      <c r="BQ19" t="s">
-        <v>199</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BQ19"/>
+  <autoFilter ref="A1:BQ18" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor(porth-import): update webhook payload structure and documentation - Modified the dispatch logic in PorthImportService to always include the purchase order ID and order number in the webhook payload, ensuring essential identifiers are sent. Additionally, updated the related documentation to reflect changes in command usage for synchronizing updated shipments.
</commit_message>
<xml_diff>
--- a/Data viva/DATA VIVA_PRUEBAS.xlsx
+++ b/Data viva/DATA VIVA_PRUEBAS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniel/Projects/Olo Orders/olo-raga-orders/Data viva/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45A6ADCD-0D31-3142-B758-4C158A1AA85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197B022B-48C4-8042-AB01-25329B339571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38040" yWindow="400" windowWidth="34200" windowHeight="21460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="750" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="201">
   <si>
     <t>ORDER_NUMBER</t>
   </si>
@@ -247,9 +247,6 @@
     <t>TRADING_COMPANY</t>
   </si>
   <si>
-    <t>Ingresada</t>
-  </si>
-  <si>
     <t>Directo CR - FERRETERIA EPA, S.A.</t>
   </si>
   <si>
@@ -307,9 +304,6 @@
     <t>( 20/11/2025 11:11:16 - LEIDY ELIETH CHAVALA : «CARGA SE ROLEO POR SOBRE PESO EN EL VAPOR 30/11/2025» )</t>
   </si>
   <si>
-    <t>Transito</t>
-  </si>
-  <si>
     <t xml:space="preserve">HANGZHOU ANAKO IMPORT AND EXPORT CO.,LTD                   </t>
   </si>
   <si>
@@ -620,19 +614,52 @@
   </si>
   <si>
     <t>OLO3</t>
+  </si>
+  <si>
+    <t>COSIARMA</t>
+  </si>
+  <si>
+    <t>SEALAND</t>
+  </si>
+  <si>
+    <t>BILBAO, SPAIN</t>
+  </si>
+  <si>
+    <t>WAIHAI, CHINA</t>
+  </si>
+  <si>
+    <t>SHANDON, CHINA</t>
+  </si>
+  <si>
+    <t>FRANKFURT, GERMANY</t>
+  </si>
+  <si>
+    <t>SHANGHAI, CHINA</t>
+  </si>
+  <si>
+    <t>NHAVA SHEVA, INDIA</t>
+  </si>
+  <si>
+    <t>BARRIOS, GUATEMALA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF2E2E2E"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -655,11 +682,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1176,57 +1204,57 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>6701122</v>
       </c>
-      <c r="B2" t="s">
-        <v>69</v>
+      <c r="B2">
+        <v>10</v>
       </c>
       <c r="C2">
         <v>865</v>
       </c>
       <c r="D2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E2">
         <v>89</v>
       </c>
       <c r="F2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G2" s="3">
         <v>9028.5</v>
       </c>
       <c r="H2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I2" s="2">
         <v>45877</v>
       </c>
       <c r="J2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K2">
         <v>2</v>
       </c>
       <c r="L2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="M2">
         <v>23</v>
       </c>
       <c r="N2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R2" s="2">
         <v>45965</v>
@@ -1241,13 +1269,13 @@
         <v>45971</v>
       </c>
       <c r="V2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W2">
         <v>26</v>
       </c>
       <c r="X2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y2" s="2">
         <v>45982</v>
@@ -1268,28 +1296,28 @@
         <v>46060</v>
       </c>
       <c r="AE2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG2">
         <v>6946</v>
       </c>
       <c r="AH2" t="s">
-        <v>84</v>
-      </c>
-      <c r="AI2">
-        <v>77</v>
+        <v>83</v>
+      </c>
+      <c r="AI2" s="4" t="s">
+        <v>194</v>
       </c>
       <c r="AJ2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK2">
-        <v>125</v>
+        <v>73</v>
+      </c>
+      <c r="AK2" s="4" t="s">
+        <v>200</v>
       </c>
       <c r="AL2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AM2" s="1">
         <v>101162</v>
@@ -1298,10 +1326,10 @@
         <v>45982</v>
       </c>
       <c r="AO2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AP2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ2" s="1">
         <v>4250</v>
@@ -1310,46 +1338,46 @@
         <v>1000001</v>
       </c>
       <c r="AS2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AU2" s="1">
         <v>9028</v>
       </c>
       <c r="AV2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AW2" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY2" t="s">
+        <v>76</v>
+      </c>
+      <c r="AZ2" t="s">
         <v>87</v>
       </c>
-      <c r="AW2" t="s">
-        <v>77</v>
-      </c>
-      <c r="AX2" t="s">
+      <c r="BA2" t="s">
+        <v>76</v>
+      </c>
+      <c r="BB2" t="s">
+        <v>76</v>
+      </c>
+      <c r="BC2" t="s">
+        <v>71</v>
+      </c>
+      <c r="BD2" t="s">
+        <v>71</v>
+      </c>
+      <c r="BE2" t="s">
         <v>78</v>
       </c>
-      <c r="AY2" t="s">
-        <v>77</v>
-      </c>
-      <c r="AZ2" t="s">
-        <v>88</v>
-      </c>
-      <c r="BA2" t="s">
-        <v>77</v>
-      </c>
-      <c r="BB2" t="s">
-        <v>77</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>72</v>
-      </c>
-      <c r="BD2" t="s">
-        <v>72</v>
-      </c>
-      <c r="BE2" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF2">
-        <v>2</v>
+      <c r="BF2" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="BG2" s="2">
         <v>45848</v>
@@ -1361,81 +1389,81 @@
         <v>0</v>
       </c>
       <c r="BJ2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="3" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>6701206</v>
       </c>
-      <c r="B3" t="s">
-        <v>89</v>
+      <c r="B3">
+        <v>5</v>
       </c>
       <c r="C3">
         <v>462</v>
       </c>
       <c r="D3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E3">
         <v>82</v>
       </c>
       <c r="F3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G3" s="3">
         <v>22127.282999999999</v>
       </c>
       <c r="H3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I3" s="2">
         <v>45883</v>
       </c>
       <c r="J3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K3">
         <v>2</v>
       </c>
       <c r="L3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="M3">
         <v>22</v>
       </c>
       <c r="N3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="O3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R3" s="2">
         <v>45982</v>
@@ -1450,13 +1478,13 @@
         <v>45989</v>
       </c>
       <c r="V3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W3">
         <v>67</v>
       </c>
       <c r="X3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y3" s="2">
         <v>46001</v>
@@ -1477,37 +1505,37 @@
         <v>46059</v>
       </c>
       <c r="AE3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG3">
         <v>7295</v>
       </c>
       <c r="AH3" t="s">
-        <v>94</v>
-      </c>
-      <c r="AI3">
-        <v>108</v>
+        <v>92</v>
+      </c>
+      <c r="AI3" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="AJ3" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK3">
-        <v>125</v>
+        <v>73</v>
+      </c>
+      <c r="AK3" s="4" t="s">
+        <v>200</v>
       </c>
       <c r="AM3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AN3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AO3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="AP3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ3" s="1">
         <v>3320</v>
@@ -1516,46 +1544,46 @@
         <v>1000001</v>
       </c>
       <c r="AS3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="AU3" s="3">
         <v>22127.279999999999</v>
       </c>
       <c r="AV3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="AW3" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX3" t="s">
         <v>77</v>
       </c>
-      <c r="AX3" t="s">
+      <c r="AY3" t="s">
+        <v>76</v>
+      </c>
+      <c r="AZ3" t="s">
+        <v>96</v>
+      </c>
+      <c r="BA3" t="s">
+        <v>76</v>
+      </c>
+      <c r="BB3" t="s">
+        <v>76</v>
+      </c>
+      <c r="BC3" t="s">
+        <v>71</v>
+      </c>
+      <c r="BD3" t="s">
+        <v>71</v>
+      </c>
+      <c r="BE3" t="s">
         <v>78</v>
       </c>
-      <c r="AY3" t="s">
-        <v>77</v>
-      </c>
-      <c r="AZ3" t="s">
-        <v>98</v>
-      </c>
-      <c r="BA3" t="s">
-        <v>77</v>
-      </c>
-      <c r="BB3" t="s">
-        <v>77</v>
-      </c>
-      <c r="BC3" t="s">
-        <v>72</v>
-      </c>
-      <c r="BD3" t="s">
-        <v>72</v>
-      </c>
-      <c r="BE3" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF3">
-        <v>8</v>
+      <c r="BF3" s="4" t="s">
+        <v>192</v>
       </c>
       <c r="BG3" s="2">
         <v>45698</v>
@@ -1567,81 +1595,81 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ3" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="4" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>6701207</v>
       </c>
-      <c r="B4" t="s">
-        <v>89</v>
+      <c r="B4">
+        <v>5</v>
       </c>
       <c r="C4">
         <v>463</v>
       </c>
       <c r="D4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E4">
         <v>82</v>
       </c>
       <c r="F4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G4" s="3">
         <v>11660.46</v>
       </c>
       <c r="H4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I4" s="2">
         <v>45883</v>
       </c>
       <c r="J4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K4">
         <v>2</v>
       </c>
       <c r="L4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="M4">
         <v>22</v>
       </c>
       <c r="N4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="O4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R4" s="2">
         <v>45982</v>
@@ -1656,13 +1684,13 @@
         <v>45989</v>
       </c>
       <c r="V4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W4">
         <v>67</v>
       </c>
       <c r="X4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y4" s="2">
         <v>46001</v>
@@ -1683,85 +1711,85 @@
         <v>46059</v>
       </c>
       <c r="AE4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG4">
         <v>7295</v>
       </c>
       <c r="AH4" t="s">
-        <v>94</v>
-      </c>
-      <c r="AI4">
-        <v>108</v>
+        <v>92</v>
+      </c>
+      <c r="AI4" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="AJ4" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK4">
-        <v>125</v>
+        <v>73</v>
+      </c>
+      <c r="AK4" s="4" t="s">
+        <v>200</v>
       </c>
       <c r="AM4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AN4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AO4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="AP4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AR4">
         <v>1000001</v>
       </c>
       <c r="AS4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="AU4" s="3">
         <v>11660.46</v>
       </c>
       <c r="AV4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="AW4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AX4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AY4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AZ4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="BA4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BB4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BC4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BD4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BE4" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF4">
-        <v>8</v>
+        <v>78</v>
+      </c>
+      <c r="BF4" s="4" t="s">
+        <v>192</v>
       </c>
       <c r="BG4" s="2">
         <v>45698</v>
@@ -1773,81 +1801,81 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ4" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="5" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>6701296</v>
       </c>
-      <c r="B5" t="s">
-        <v>69</v>
+      <c r="B5">
+        <v>10</v>
       </c>
       <c r="C5">
         <v>904</v>
       </c>
       <c r="D5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E5">
         <v>82</v>
       </c>
       <c r="F5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G5" s="3">
         <v>26948.92</v>
       </c>
       <c r="H5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I5" s="2">
         <v>45890</v>
       </c>
       <c r="J5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K5">
         <v>2</v>
       </c>
       <c r="L5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="M5">
         <v>22</v>
       </c>
       <c r="N5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="O5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R5" s="2">
         <v>45968</v>
@@ -1862,13 +1890,13 @@
         <v>45991</v>
       </c>
       <c r="V5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W5">
         <v>54</v>
       </c>
       <c r="X5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y5" s="2">
         <v>45991</v>
@@ -1889,28 +1917,28 @@
         <v>46060</v>
       </c>
       <c r="AE5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG5">
         <v>7156</v>
       </c>
       <c r="AH5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AI5" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK5" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="AL5" t="s">
         <v>75</v>
-      </c>
-      <c r="AI5">
-        <v>91</v>
-      </c>
-      <c r="AJ5" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK5">
-        <v>125</v>
-      </c>
-      <c r="AL5" t="s">
-        <v>76</v>
       </c>
       <c r="AM5" s="1">
         <v>101367</v>
@@ -1919,10 +1947,10 @@
         <v>46003</v>
       </c>
       <c r="AO5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AP5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ5" s="1">
         <v>4250</v>
@@ -1931,46 +1959,46 @@
         <v>1000001</v>
       </c>
       <c r="AS5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="AU5" s="3">
         <v>26948.92</v>
       </c>
       <c r="AV5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="AW5" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX5" t="s">
         <v>77</v>
       </c>
-      <c r="AX5" t="s">
-        <v>78</v>
-      </c>
       <c r="AY5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AZ5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BA5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BB5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BC5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BD5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BE5" t="s">
-        <v>107</v>
-      </c>
-      <c r="BF5">
-        <v>2</v>
+        <v>105</v>
+      </c>
+      <c r="BF5" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="BG5" s="2">
         <v>45848</v>
@@ -1982,81 +2010,81 @@
         <v>0</v>
       </c>
       <c r="BJ5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="6" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>6701297</v>
       </c>
-      <c r="B6" t="s">
-        <v>69</v>
+      <c r="B6">
+        <v>10</v>
       </c>
       <c r="C6">
         <v>904</v>
       </c>
       <c r="D6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E6">
         <v>82</v>
       </c>
       <c r="F6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G6" s="3">
         <v>26985.119999999999</v>
       </c>
       <c r="H6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I6" s="2">
         <v>45890</v>
       </c>
       <c r="J6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K6">
         <v>2</v>
       </c>
       <c r="L6" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="M6">
         <v>22</v>
       </c>
       <c r="N6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="O6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R6" s="2">
         <v>45968</v>
@@ -2071,13 +2099,13 @@
         <v>45989</v>
       </c>
       <c r="V6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W6">
         <v>52</v>
       </c>
       <c r="X6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y6" s="2">
         <v>45991</v>
@@ -2098,28 +2126,28 @@
         <v>46060</v>
       </c>
       <c r="AE6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG6">
         <v>7150</v>
       </c>
       <c r="AH6" t="s">
+        <v>74</v>
+      </c>
+      <c r="AI6" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK6" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="AL6" t="s">
         <v>75</v>
-      </c>
-      <c r="AI6">
-        <v>91</v>
-      </c>
-      <c r="AJ6" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK6">
-        <v>125</v>
-      </c>
-      <c r="AL6" t="s">
-        <v>76</v>
       </c>
       <c r="AM6" s="1">
         <v>101358</v>
@@ -2128,10 +2156,10 @@
         <v>46002</v>
       </c>
       <c r="AO6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AP6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ6" s="1">
         <v>4250</v>
@@ -2140,46 +2168,46 @@
         <v>1000001</v>
       </c>
       <c r="AS6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT6" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="AU6" s="3">
         <v>26985.119999999999</v>
       </c>
       <c r="AV6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AW6" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX6" t="s">
         <v>77</v>
       </c>
-      <c r="AX6" t="s">
-        <v>78</v>
-      </c>
       <c r="AY6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AZ6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BA6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BB6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BC6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BD6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BE6" t="s">
-        <v>107</v>
-      </c>
-      <c r="BF6">
-        <v>2</v>
+        <v>105</v>
+      </c>
+      <c r="BF6" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="BG6" s="2">
         <v>45848</v>
@@ -2191,81 +2219,81 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="7" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6701353</v>
       </c>
-      <c r="B7" t="s">
-        <v>69</v>
+      <c r="B7">
+        <v>10</v>
       </c>
       <c r="C7">
         <v>270</v>
       </c>
       <c r="D7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E7">
         <v>88</v>
       </c>
       <c r="F7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G7" s="1">
         <v>17712</v>
       </c>
       <c r="H7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I7" s="2">
         <v>45897</v>
       </c>
       <c r="J7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K7">
         <v>2</v>
       </c>
       <c r="L7" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="M7">
         <v>23</v>
       </c>
       <c r="N7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="O7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R7" s="2">
         <v>45974</v>
@@ -2280,13 +2308,13 @@
         <v>45975</v>
       </c>
       <c r="V7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W7">
         <v>30</v>
       </c>
       <c r="X7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y7" s="2">
         <v>45984</v>
@@ -2307,28 +2335,28 @@
         <v>46060</v>
       </c>
       <c r="AE7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG7">
         <v>7207</v>
       </c>
       <c r="AH7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AI7" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK7" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="AL7" t="s">
         <v>75</v>
-      </c>
-      <c r="AI7">
-        <v>91</v>
-      </c>
-      <c r="AJ7" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK7">
-        <v>125</v>
-      </c>
-      <c r="AL7" t="s">
-        <v>76</v>
       </c>
       <c r="AM7" s="1">
         <v>101433</v>
@@ -2337,10 +2365,10 @@
         <v>46009</v>
       </c>
       <c r="AO7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="AP7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ7" s="1">
         <v>3320</v>
@@ -2349,46 +2377,46 @@
         <v>1000001</v>
       </c>
       <c r="AS7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT7" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="AU7" s="1">
         <v>17712</v>
       </c>
       <c r="AV7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AW7" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX7" t="s">
         <v>77</v>
       </c>
-      <c r="AX7" t="s">
+      <c r="AY7" t="s">
+        <v>73</v>
+      </c>
+      <c r="AZ7" t="s">
+        <v>116</v>
+      </c>
+      <c r="BA7" t="s">
+        <v>76</v>
+      </c>
+      <c r="BB7" t="s">
+        <v>76</v>
+      </c>
+      <c r="BC7" t="s">
+        <v>71</v>
+      </c>
+      <c r="BD7" t="s">
+        <v>71</v>
+      </c>
+      <c r="BE7" t="s">
         <v>78</v>
       </c>
-      <c r="AY7" t="s">
-        <v>74</v>
-      </c>
-      <c r="AZ7" t="s">
-        <v>118</v>
-      </c>
-      <c r="BA7" t="s">
-        <v>77</v>
-      </c>
-      <c r="BB7" t="s">
-        <v>77</v>
-      </c>
-      <c r="BC7" t="s">
-        <v>72</v>
-      </c>
-      <c r="BD7" t="s">
-        <v>72</v>
-      </c>
-      <c r="BE7" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF7">
-        <v>2</v>
+      <c r="BF7" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="BG7" s="2">
         <v>45848</v>
@@ -2400,81 +2428,81 @@
         <v>0</v>
       </c>
       <c r="BJ7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="8" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>6701683</v>
       </c>
-      <c r="B8" t="s">
-        <v>69</v>
+      <c r="B8">
+        <v>10</v>
       </c>
       <c r="C8">
         <v>380</v>
       </c>
       <c r="D8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E8">
         <v>85</v>
       </c>
       <c r="F8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G8" s="3">
         <v>20570.05</v>
       </c>
       <c r="H8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I8" s="2">
         <v>45911</v>
       </c>
       <c r="J8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K8">
         <v>2</v>
       </c>
       <c r="L8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="M8">
         <v>23</v>
       </c>
       <c r="N8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="O8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R8" s="2">
         <v>45964</v>
@@ -2489,13 +2517,13 @@
         <v>45976</v>
       </c>
       <c r="V8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W8">
         <v>0</v>
       </c>
       <c r="X8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y8" s="2">
         <v>45983</v>
@@ -2516,28 +2544,28 @@
         <v>46060</v>
       </c>
       <c r="AE8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG8">
         <v>7130</v>
       </c>
       <c r="AH8" t="s">
+        <v>74</v>
+      </c>
+      <c r="AI8" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="AJ8" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK8" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="AL8" t="s">
         <v>75</v>
-      </c>
-      <c r="AI8">
-        <v>77</v>
-      </c>
-      <c r="AJ8" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK8">
-        <v>125</v>
-      </c>
-      <c r="AL8" t="s">
-        <v>76</v>
       </c>
       <c r="AM8" s="1">
         <v>101335</v>
@@ -2546,10 +2574,10 @@
         <v>46001</v>
       </c>
       <c r="AO8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="AP8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ8" s="1">
         <v>4290</v>
@@ -2558,49 +2586,49 @@
         <v>1000024</v>
       </c>
       <c r="AS8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT8" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="AU8" s="3">
         <v>20570.05</v>
       </c>
       <c r="AV8" t="s">
+        <v>122</v>
+      </c>
+      <c r="AW8" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX8" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY8" t="s">
+        <v>73</v>
+      </c>
+      <c r="AZ8" t="s">
+        <v>123</v>
+      </c>
+      <c r="BA8" t="s">
+        <v>76</v>
+      </c>
+      <c r="BB8" t="s">
+        <v>76</v>
+      </c>
+      <c r="BC8" t="s">
+        <v>71</v>
+      </c>
+      <c r="BD8" t="s">
+        <v>71</v>
+      </c>
+      <c r="BE8" t="s">
+        <v>78</v>
+      </c>
+      <c r="BF8" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="BG8" t="s">
         <v>124</v>
-      </c>
-      <c r="AW8" t="s">
-        <v>77</v>
-      </c>
-      <c r="AX8" t="s">
-        <v>78</v>
-      </c>
-      <c r="AY8" t="s">
-        <v>74</v>
-      </c>
-      <c r="AZ8" t="s">
-        <v>125</v>
-      </c>
-      <c r="BA8" t="s">
-        <v>77</v>
-      </c>
-      <c r="BB8" t="s">
-        <v>77</v>
-      </c>
-      <c r="BC8" t="s">
-        <v>72</v>
-      </c>
-      <c r="BD8" t="s">
-        <v>72</v>
-      </c>
-      <c r="BE8" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF8">
-        <v>2</v>
-      </c>
-      <c r="BG8" t="s">
-        <v>126</v>
       </c>
       <c r="BH8">
         <v>14</v>
@@ -2609,81 +2637,81 @@
         <v>0</v>
       </c>
       <c r="BJ8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="9" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>6701684</v>
       </c>
-      <c r="B9" t="s">
-        <v>69</v>
+      <c r="B9">
+        <v>10</v>
       </c>
       <c r="C9">
         <v>380</v>
       </c>
       <c r="D9" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E9">
         <v>85</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G9" s="3">
         <v>20570.05</v>
       </c>
       <c r="H9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I9" s="2">
         <v>45911</v>
       </c>
       <c r="J9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K9">
         <v>2</v>
       </c>
       <c r="L9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="M9">
         <v>23</v>
       </c>
       <c r="N9" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="O9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R9" s="2">
         <v>45964</v>
@@ -2698,13 +2726,13 @@
         <v>45976</v>
       </c>
       <c r="V9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W9">
         <v>0</v>
       </c>
       <c r="X9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y9" s="2">
         <v>45982</v>
@@ -2725,28 +2753,28 @@
         <v>46060</v>
       </c>
       <c r="AE9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG9">
         <v>7132</v>
       </c>
       <c r="AH9" t="s">
+        <v>74</v>
+      </c>
+      <c r="AI9" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="AJ9" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK9" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="AL9" t="s">
         <v>75</v>
-      </c>
-      <c r="AI9">
-        <v>77</v>
-      </c>
-      <c r="AJ9" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK9">
-        <v>125</v>
-      </c>
-      <c r="AL9" t="s">
-        <v>76</v>
       </c>
       <c r="AM9" s="1">
         <v>101337</v>
@@ -2755,10 +2783,10 @@
         <v>46001</v>
       </c>
       <c r="AO9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="AP9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ9" s="1">
         <v>4190</v>
@@ -2767,49 +2795,49 @@
         <v>1000024</v>
       </c>
       <c r="AS9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="AU9" s="3">
         <v>20570.05</v>
       </c>
       <c r="AV9" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="AW9" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX9" t="s">
         <v>77</v>
       </c>
-      <c r="AX9" t="s">
+      <c r="AY9" t="s">
+        <v>73</v>
+      </c>
+      <c r="AZ9" t="s">
+        <v>130</v>
+      </c>
+      <c r="BA9" t="s">
+        <v>76</v>
+      </c>
+      <c r="BB9" t="s">
+        <v>76</v>
+      </c>
+      <c r="BC9" t="s">
+        <v>71</v>
+      </c>
+      <c r="BD9" t="s">
+        <v>71</v>
+      </c>
+      <c r="BE9" t="s">
         <v>78</v>
       </c>
-      <c r="AY9" t="s">
-        <v>74</v>
-      </c>
-      <c r="AZ9" t="s">
-        <v>132</v>
-      </c>
-      <c r="BA9" t="s">
-        <v>77</v>
-      </c>
-      <c r="BB9" t="s">
-        <v>77</v>
-      </c>
-      <c r="BC9" t="s">
-        <v>72</v>
-      </c>
-      <c r="BD9" t="s">
-        <v>72</v>
-      </c>
-      <c r="BE9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF9">
-        <v>2</v>
+      <c r="BF9" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="BG9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="BH9">
         <v>14</v>
@@ -2818,81 +2846,81 @@
         <v>0</v>
       </c>
       <c r="BJ9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ9" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="10" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>6701758</v>
       </c>
-      <c r="B10" t="s">
-        <v>89</v>
+      <c r="B10">
+        <v>5</v>
       </c>
       <c r="C10">
         <v>903</v>
       </c>
       <c r="D10" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E10">
         <v>85</v>
       </c>
       <c r="F10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G10" s="3">
         <v>29145.119999999999</v>
       </c>
       <c r="H10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I10" s="2">
         <v>45922</v>
       </c>
       <c r="J10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K10">
         <v>2</v>
       </c>
       <c r="L10" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="M10">
         <v>23</v>
       </c>
       <c r="N10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="O10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R10" s="2">
         <v>45982</v>
@@ -2907,13 +2935,13 @@
         <v>45985</v>
       </c>
       <c r="V10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W10">
         <v>-1</v>
       </c>
       <c r="X10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y10" s="2">
         <v>45991</v>
@@ -2934,37 +2962,37 @@
         <v>46060</v>
       </c>
       <c r="AE10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG10">
         <v>7245</v>
       </c>
       <c r="AH10" t="s">
-        <v>94</v>
-      </c>
-      <c r="AI10">
-        <v>36</v>
+        <v>92</v>
+      </c>
+      <c r="AI10" s="4" t="s">
+        <v>197</v>
       </c>
       <c r="AJ10" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK10">
-        <v>125</v>
+        <v>73</v>
+      </c>
+      <c r="AK10" s="4" t="s">
+        <v>200</v>
       </c>
       <c r="AM10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AN10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AO10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AP10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ10" s="1">
         <v>4715</v>
@@ -2973,46 +3001,46 @@
         <v>1000001</v>
       </c>
       <c r="AS10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="AU10" s="3">
         <v>29145.119999999999</v>
       </c>
       <c r="AV10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AW10" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX10" t="s">
         <v>77</v>
       </c>
-      <c r="AX10" t="s">
+      <c r="AY10" t="s">
+        <v>76</v>
+      </c>
+      <c r="AZ10" t="s">
+        <v>137</v>
+      </c>
+      <c r="BA10" t="s">
+        <v>73</v>
+      </c>
+      <c r="BB10" t="s">
+        <v>76</v>
+      </c>
+      <c r="BC10" t="s">
+        <v>71</v>
+      </c>
+      <c r="BD10" t="s">
+        <v>71</v>
+      </c>
+      <c r="BE10" t="s">
         <v>78</v>
       </c>
-      <c r="AY10" t="s">
-        <v>77</v>
-      </c>
-      <c r="AZ10" t="s">
-        <v>139</v>
-      </c>
-      <c r="BA10" t="s">
-        <v>74</v>
-      </c>
-      <c r="BB10" t="s">
-        <v>77</v>
-      </c>
-      <c r="BC10" t="s">
-        <v>72</v>
-      </c>
-      <c r="BD10" t="s">
-        <v>72</v>
-      </c>
-      <c r="BE10" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF10">
-        <v>2</v>
+      <c r="BF10" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="BG10" s="2">
         <v>45972</v>
@@ -3024,81 +3052,81 @@
         <v>0</v>
       </c>
       <c r="BJ10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ10" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="11" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>6701769</v>
       </c>
-      <c r="B11" t="s">
-        <v>69</v>
+      <c r="B11">
+        <v>10</v>
       </c>
       <c r="C11">
         <v>905</v>
       </c>
       <c r="D11" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E11">
         <v>89</v>
       </c>
       <c r="F11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G11" s="1">
         <v>13860</v>
       </c>
       <c r="H11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I11" s="2">
         <v>45923</v>
       </c>
       <c r="J11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K11">
         <v>2</v>
       </c>
       <c r="L11" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M11">
         <v>23</v>
       </c>
       <c r="N11" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="O11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R11" s="2">
         <v>45975</v>
@@ -3113,13 +3141,13 @@
         <v>45986</v>
       </c>
       <c r="V11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W11">
         <v>7</v>
       </c>
       <c r="X11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y11" s="2">
         <v>45994</v>
@@ -3140,28 +3168,28 @@
         <v>46060</v>
       </c>
       <c r="AE11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG11">
         <v>7103</v>
       </c>
       <c r="AH11" t="s">
+        <v>74</v>
+      </c>
+      <c r="AI11" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="AJ11" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK11" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="AL11" t="s">
         <v>75</v>
-      </c>
-      <c r="AI11">
-        <v>108</v>
-      </c>
-      <c r="AJ11" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK11">
-        <v>125</v>
-      </c>
-      <c r="AL11" t="s">
-        <v>76</v>
       </c>
       <c r="AM11" s="1">
         <v>101298</v>
@@ -3170,10 +3198,10 @@
         <v>45999</v>
       </c>
       <c r="AO11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="AP11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ11" s="1">
         <v>4250</v>
@@ -3182,49 +3210,49 @@
         <v>1000001</v>
       </c>
       <c r="AS11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT11" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="AU11" s="1">
         <v>13860</v>
       </c>
       <c r="AV11" t="s">
+        <v>143</v>
+      </c>
+      <c r="AW11" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX11" t="s">
+        <v>144</v>
+      </c>
+      <c r="AY11" t="s">
+        <v>76</v>
+      </c>
+      <c r="AZ11" t="s">
+        <v>71</v>
+      </c>
+      <c r="BA11" t="s">
+        <v>76</v>
+      </c>
+      <c r="BB11" t="s">
+        <v>76</v>
+      </c>
+      <c r="BC11" t="s">
+        <v>71</v>
+      </c>
+      <c r="BD11" t="s">
+        <v>71</v>
+      </c>
+      <c r="BE11" t="s">
+        <v>78</v>
+      </c>
+      <c r="BF11" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="BG11" t="s">
         <v>145</v>
-      </c>
-      <c r="AW11" t="s">
-        <v>77</v>
-      </c>
-      <c r="AX11" t="s">
-        <v>146</v>
-      </c>
-      <c r="AY11" t="s">
-        <v>77</v>
-      </c>
-      <c r="AZ11" t="s">
-        <v>72</v>
-      </c>
-      <c r="BA11" t="s">
-        <v>77</v>
-      </c>
-      <c r="BB11" t="s">
-        <v>77</v>
-      </c>
-      <c r="BC11" t="s">
-        <v>72</v>
-      </c>
-      <c r="BD11" t="s">
-        <v>72</v>
-      </c>
-      <c r="BE11" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF11">
-        <v>2</v>
-      </c>
-      <c r="BG11" t="s">
-        <v>147</v>
       </c>
       <c r="BH11">
         <v>14</v>
@@ -3233,81 +3261,81 @@
         <v>0</v>
       </c>
       <c r="BJ11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ11" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="12" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>6701770</v>
       </c>
-      <c r="B12" t="s">
-        <v>89</v>
+      <c r="B12">
+        <v>5</v>
       </c>
       <c r="C12">
         <v>905</v>
       </c>
       <c r="D12" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E12">
         <v>89</v>
       </c>
       <c r="F12" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G12" s="1">
         <v>5841</v>
       </c>
       <c r="H12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I12" s="2">
         <v>45923</v>
       </c>
       <c r="J12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K12">
         <v>2</v>
       </c>
       <c r="L12" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="M12">
         <v>23</v>
       </c>
       <c r="N12" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="O12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R12" s="2">
         <v>45975</v>
@@ -3322,13 +3350,13 @@
         <v>45986</v>
       </c>
       <c r="V12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W12">
         <v>7</v>
       </c>
       <c r="X12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y12" s="2">
         <v>45994</v>
@@ -3349,88 +3377,88 @@
         <v>46060</v>
       </c>
       <c r="AE12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG12">
         <v>7190</v>
       </c>
       <c r="AH12" t="s">
-        <v>94</v>
-      </c>
-      <c r="AI12">
-        <v>108</v>
+        <v>92</v>
+      </c>
+      <c r="AI12" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="AJ12" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK12">
-        <v>125</v>
+        <v>73</v>
+      </c>
+      <c r="AK12" s="4" t="s">
+        <v>200</v>
       </c>
       <c r="AM12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AN12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AO12" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="AP12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AR12">
         <v>1000001</v>
       </c>
       <c r="AS12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="AU12" s="1">
         <v>5841</v>
       </c>
       <c r="AV12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="AW12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AX12" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="AY12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AZ12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BA12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BB12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BC12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BD12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BE12" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF12">
-        <v>2</v>
+        <v>78</v>
+      </c>
+      <c r="BF12" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="BG12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="BH12">
         <v>14</v>
@@ -3439,81 +3467,81 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ12" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="13" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>6701771</v>
       </c>
-      <c r="B13" t="s">
-        <v>69</v>
+      <c r="B13">
+        <v>10</v>
       </c>
       <c r="C13">
         <v>905</v>
       </c>
       <c r="D13" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E13">
         <v>89</v>
       </c>
       <c r="F13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G13" s="1">
         <v>2720</v>
       </c>
       <c r="H13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I13" s="2">
         <v>45923</v>
       </c>
       <c r="J13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K13">
         <v>2</v>
       </c>
       <c r="L13" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="M13">
         <v>23</v>
       </c>
       <c r="N13" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="O13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R13" s="2">
         <v>45975</v>
@@ -3528,13 +3556,13 @@
         <v>45986</v>
       </c>
       <c r="V13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W13">
         <v>7</v>
       </c>
       <c r="X13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y13" s="2">
         <v>45994</v>
@@ -3555,28 +3583,28 @@
         <v>46060</v>
       </c>
       <c r="AE13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG13">
         <v>7104</v>
       </c>
       <c r="AH13" t="s">
+        <v>74</v>
+      </c>
+      <c r="AI13" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="AJ13" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK13" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="AL13" t="s">
         <v>75</v>
-      </c>
-      <c r="AI13">
-        <v>108</v>
-      </c>
-      <c r="AJ13" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK13">
-        <v>125</v>
-      </c>
-      <c r="AL13" t="s">
-        <v>76</v>
       </c>
       <c r="AM13" s="1">
         <v>101299</v>
@@ -3585,10 +3613,10 @@
         <v>45999</v>
       </c>
       <c r="AO13" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ13" s="1">
         <v>3320</v>
@@ -3597,49 +3625,49 @@
         <v>1000001</v>
       </c>
       <c r="AS13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT13" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="AU13" s="1">
         <v>2720</v>
       </c>
       <c r="AV13" t="s">
+        <v>155</v>
+      </c>
+      <c r="AW13" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX13" t="s">
+        <v>156</v>
+      </c>
+      <c r="AY13" t="s">
+        <v>76</v>
+      </c>
+      <c r="AZ13" t="s">
         <v>157</v>
       </c>
-      <c r="AW13" t="s">
-        <v>77</v>
-      </c>
-      <c r="AX13" t="s">
-        <v>158</v>
-      </c>
-      <c r="AY13" t="s">
-        <v>77</v>
-      </c>
-      <c r="AZ13" t="s">
-        <v>159</v>
-      </c>
       <c r="BA13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BB13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BC13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BD13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BE13" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF13">
-        <v>2</v>
+        <v>78</v>
+      </c>
+      <c r="BF13" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="BG13" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="BH13">
         <v>14</v>
@@ -3648,81 +3676,81 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ13" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="14" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>6701772</v>
       </c>
-      <c r="B14" t="s">
-        <v>89</v>
+      <c r="B14">
+        <v>5</v>
       </c>
       <c r="C14">
         <v>905</v>
       </c>
       <c r="D14" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E14">
         <v>89</v>
       </c>
       <c r="F14" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G14" s="1">
         <v>18305</v>
       </c>
       <c r="H14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I14" s="2">
         <v>45923</v>
       </c>
       <c r="J14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K14">
         <v>2</v>
       </c>
       <c r="L14" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="M14">
         <v>23</v>
       </c>
       <c r="N14" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="O14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R14" s="2">
         <v>45975</v>
@@ -3737,13 +3765,13 @@
         <v>45985</v>
       </c>
       <c r="V14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W14">
         <v>6</v>
       </c>
       <c r="X14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y14" s="2">
         <v>45994</v>
@@ -3764,88 +3792,88 @@
         <v>46060</v>
       </c>
       <c r="AE14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG14">
         <v>7227</v>
       </c>
       <c r="AH14" t="s">
-        <v>94</v>
-      </c>
-      <c r="AI14">
-        <v>108</v>
+        <v>92</v>
+      </c>
+      <c r="AI14" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="AJ14" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK14">
-        <v>125</v>
+        <v>73</v>
+      </c>
+      <c r="AK14" s="4" t="s">
+        <v>200</v>
       </c>
       <c r="AM14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AN14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AO14" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="AP14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AR14">
         <v>1000001</v>
       </c>
       <c r="AS14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT14" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="AU14" s="1">
         <v>18305</v>
       </c>
       <c r="AV14" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AW14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AX14" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="AY14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AZ14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BA14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BB14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BC14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BD14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BE14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF14">
-        <v>2</v>
+        <v>78</v>
+      </c>
+      <c r="BF14" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="BG14" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="BH14">
         <v>14</v>
@@ -3854,81 +3882,81 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ14" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="15" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>6702103</v>
       </c>
-      <c r="B15" t="s">
-        <v>69</v>
+      <c r="B15">
+        <v>10</v>
       </c>
       <c r="C15">
         <v>913</v>
       </c>
       <c r="D15" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E15">
         <v>85</v>
       </c>
       <c r="F15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G15" s="1">
         <v>13090</v>
       </c>
       <c r="H15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I15" s="2">
         <v>45951</v>
       </c>
       <c r="J15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K15">
         <v>2</v>
       </c>
       <c r="L15" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="M15">
         <v>23</v>
       </c>
       <c r="N15" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="O15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R15" s="2">
         <v>45994</v>
@@ -3943,13 +3971,13 @@
         <v>45991</v>
       </c>
       <c r="V15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W15">
         <v>-8</v>
       </c>
       <c r="X15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y15" s="2">
         <v>46003</v>
@@ -3970,28 +3998,28 @@
         <v>46060</v>
       </c>
       <c r="AE15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG15">
         <v>7192</v>
       </c>
       <c r="AH15" t="s">
+        <v>74</v>
+      </c>
+      <c r="AI15" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="AJ15" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK15" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="AL15" t="s">
         <v>75</v>
-      </c>
-      <c r="AI15">
-        <v>92</v>
-      </c>
-      <c r="AJ15" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK15">
-        <v>125</v>
-      </c>
-      <c r="AL15" t="s">
-        <v>76</v>
       </c>
       <c r="AM15" s="1">
         <v>101418</v>
@@ -4000,10 +4028,10 @@
         <v>46008</v>
       </c>
       <c r="AO15" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="AP15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ15" s="1">
         <v>3125</v>
@@ -4012,46 +4040,46 @@
         <v>1000007</v>
       </c>
       <c r="AS15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT15" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="AU15" s="1">
         <v>13090</v>
       </c>
       <c r="AV15" t="s">
+        <v>168</v>
+      </c>
+      <c r="AW15" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX15" t="s">
+        <v>169</v>
+      </c>
+      <c r="AY15" t="s">
+        <v>76</v>
+      </c>
+      <c r="AZ15" t="s">
         <v>170</v>
       </c>
-      <c r="AW15" t="s">
-        <v>77</v>
-      </c>
-      <c r="AX15" t="s">
-        <v>171</v>
-      </c>
-      <c r="AY15" t="s">
-        <v>77</v>
-      </c>
-      <c r="AZ15" t="s">
-        <v>172</v>
-      </c>
       <c r="BA15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BB15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BC15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BD15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BE15" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF15">
-        <v>2</v>
+        <v>78</v>
+      </c>
+      <c r="BF15" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="BG15" s="2">
         <v>45700</v>
@@ -4063,81 +4091,81 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ15" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="16" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>6702104</v>
       </c>
-      <c r="B16" t="s">
-        <v>89</v>
+      <c r="B16">
+        <v>5</v>
       </c>
       <c r="C16">
         <v>913</v>
       </c>
       <c r="D16" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E16">
         <v>85</v>
       </c>
       <c r="F16" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G16" s="1">
         <v>5950</v>
       </c>
       <c r="H16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I16" s="2">
         <v>45951</v>
       </c>
       <c r="J16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K16">
         <v>2</v>
       </c>
       <c r="L16" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="M16">
         <v>23</v>
       </c>
       <c r="N16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="O16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R16" s="2">
         <v>45994</v>
@@ -4152,13 +4180,13 @@
         <v>45991</v>
       </c>
       <c r="V16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W16">
         <v>-8</v>
       </c>
       <c r="X16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y16" s="2">
         <v>46003</v>
@@ -4179,85 +4207,85 @@
         <v>46060</v>
       </c>
       <c r="AE16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG16">
         <v>7461</v>
       </c>
       <c r="AH16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AI16">
         <v>92</v>
       </c>
+      <c r="AI16" s="4" t="s">
+        <v>198</v>
+      </c>
       <c r="AJ16" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK16">
-        <v>125</v>
+        <v>73</v>
+      </c>
+      <c r="AK16" s="4" t="s">
+        <v>200</v>
       </c>
       <c r="AM16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AN16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AO16" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="AP16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AR16">
         <v>1000007</v>
       </c>
       <c r="AS16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT16" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="AU16" s="1">
         <v>5950</v>
       </c>
       <c r="AV16" t="s">
+        <v>174</v>
+      </c>
+      <c r="AW16" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX16" t="s">
+        <v>175</v>
+      </c>
+      <c r="AY16" t="s">
+        <v>76</v>
+      </c>
+      <c r="AZ16" t="s">
         <v>176</v>
       </c>
-      <c r="AW16" t="s">
-        <v>77</v>
-      </c>
-      <c r="AX16" t="s">
-        <v>177</v>
-      </c>
-      <c r="AY16" t="s">
-        <v>77</v>
-      </c>
-      <c r="AZ16" t="s">
-        <v>178</v>
-      </c>
       <c r="BA16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BB16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BC16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BD16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BE16" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF16">
-        <v>2</v>
+        <v>78</v>
+      </c>
+      <c r="BF16" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="BG16" s="2">
         <v>45700</v>
@@ -4269,81 +4297,81 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ16" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="17" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>6702106</v>
       </c>
-      <c r="B17" t="s">
-        <v>69</v>
+      <c r="B17">
+        <v>10</v>
       </c>
       <c r="C17">
         <v>494</v>
       </c>
       <c r="D17" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E17">
         <v>83</v>
       </c>
       <c r="F17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G17" s="3">
         <v>22673.74</v>
       </c>
       <c r="H17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I17" s="2">
         <v>45951</v>
       </c>
       <c r="J17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K17">
         <v>2</v>
       </c>
       <c r="L17" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="M17">
         <v>21</v>
       </c>
       <c r="N17" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="O17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R17" s="2">
         <v>45979</v>
@@ -4358,13 +4386,13 @@
         <v>45983</v>
       </c>
       <c r="V17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W17">
         <v>-18</v>
       </c>
       <c r="X17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y17" s="2">
         <v>46001</v>
@@ -4385,28 +4413,28 @@
         <v>46059</v>
       </c>
       <c r="AE17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG17">
         <v>7510</v>
       </c>
       <c r="AH17" t="s">
+        <v>74</v>
+      </c>
+      <c r="AI17" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="AJ17" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK17" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="AL17" t="s">
         <v>75</v>
-      </c>
-      <c r="AI17">
-        <v>71</v>
-      </c>
-      <c r="AJ17" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK17">
-        <v>125</v>
-      </c>
-      <c r="AL17" t="s">
-        <v>76</v>
       </c>
       <c r="AM17" s="1">
         <v>101761</v>
@@ -4415,10 +4443,10 @@
         <v>46055</v>
       </c>
       <c r="AO17" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="AP17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ17" s="1">
         <v>3320</v>
@@ -4427,46 +4455,46 @@
         <v>1000001</v>
       </c>
       <c r="AS17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT17" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="AU17" s="3">
         <v>22673.74</v>
       </c>
       <c r="AV17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="AW17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AX17" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="AY17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AZ17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BA17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BB17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BC17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BD17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BE17" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF17">
-        <v>8</v>
+        <v>78</v>
+      </c>
+      <c r="BF17" s="4" t="s">
+        <v>192</v>
       </c>
       <c r="BG17" s="2">
         <v>45819</v>
@@ -4478,81 +4506,81 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ17" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
-    <row r="18" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:69" ht="18" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>6702107</v>
       </c>
-      <c r="B18" t="s">
-        <v>89</v>
+      <c r="B18">
+        <v>5</v>
       </c>
       <c r="C18">
         <v>494</v>
       </c>
       <c r="D18" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E18">
         <v>83</v>
       </c>
       <c r="F18" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G18" s="3">
         <v>58880.98</v>
       </c>
       <c r="H18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I18" s="2">
         <v>45951</v>
       </c>
       <c r="J18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K18">
         <v>2</v>
       </c>
       <c r="L18" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="M18">
         <v>25</v>
       </c>
       <c r="N18" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="O18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R18" s="2">
         <v>45979</v>
@@ -4567,13 +4595,13 @@
         <v>45983</v>
       </c>
       <c r="V18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W18">
         <v>-18</v>
       </c>
       <c r="X18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y18" s="2">
         <v>46001</v>
@@ -4594,85 +4622,85 @@
         <v>46059</v>
       </c>
       <c r="AE18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AG18">
         <v>7474</v>
       </c>
       <c r="AH18" t="s">
-        <v>94</v>
-      </c>
-      <c r="AI18">
-        <v>71</v>
+        <v>92</v>
+      </c>
+      <c r="AI18" s="4" t="s">
+        <v>199</v>
       </c>
       <c r="AJ18" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK18">
-        <v>125</v>
+        <v>73</v>
+      </c>
+      <c r="AK18" s="4" t="s">
+        <v>200</v>
       </c>
       <c r="AM18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AN18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AO18" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="AP18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AR18">
         <v>1000001</v>
       </c>
       <c r="AS18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AT18" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="AU18" s="3">
         <v>58880.98</v>
       </c>
       <c r="AV18" t="s">
+        <v>187</v>
+      </c>
+      <c r="AW18" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX18" t="s">
+        <v>188</v>
+      </c>
+      <c r="AY18" t="s">
+        <v>76</v>
+      </c>
+      <c r="AZ18" t="s">
         <v>189</v>
       </c>
-      <c r="AW18" t="s">
-        <v>77</v>
-      </c>
-      <c r="AX18" t="s">
+      <c r="BA18" t="s">
+        <v>76</v>
+      </c>
+      <c r="BB18" t="s">
+        <v>76</v>
+      </c>
+      <c r="BC18" t="s">
+        <v>71</v>
+      </c>
+      <c r="BD18" t="s">
+        <v>71</v>
+      </c>
+      <c r="BE18" t="s">
         <v>190</v>
       </c>
-      <c r="AY18" t="s">
-        <v>77</v>
-      </c>
-      <c r="AZ18" t="s">
-        <v>191</v>
-      </c>
-      <c r="BA18" t="s">
-        <v>77</v>
-      </c>
-      <c r="BB18" t="s">
-        <v>77</v>
-      </c>
-      <c r="BC18" t="s">
-        <v>72</v>
-      </c>
-      <c r="BD18" t="s">
-        <v>72</v>
-      </c>
-      <c r="BE18" t="s">
+      <c r="BF18" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="BF18">
-        <v>8</v>
       </c>
       <c r="BG18" s="2">
         <v>45819</v>
@@ -4684,28 +4712,28 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BK18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BL18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BM18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BN18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BO18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BP18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BQ18" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data-management): remove temporary Excel file and update CSV data - Deleted the temporary Excel file used for testing and updated the CSV file with new shipping data, including changes to vendor names and shipping details for improved accuracy in reporting. Additionally, modified the dashboard views to reflect updated filter descriptions for better clarity.
</commit_message>
<xml_diff>
--- a/Data viva/DATA VIVA_PRUEBAS.xlsx
+++ b/Data viva/DATA VIVA_PRUEBAS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniel/Projects/Olo Orders/olo-raga-orders/Data viva/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197B022B-48C4-8042-AB01-25329B339571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D60A84F2-DC9C-254C-9DF4-C810F78FAACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38040" yWindow="400" windowWidth="34200" windowHeight="21460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="196">
   <si>
     <t>ORDER_NUMBER</t>
   </si>
@@ -343,9 +343,6 @@
     <t>INTCO INTERNATIONAL(HK) CO., LIMITED 2</t>
   </si>
   <si>
-    <t>ASSHA510643</t>
-  </si>
-  <si>
     <t>MSMU5604550</t>
   </si>
   <si>
@@ -358,9 +355,6 @@
     <t>PEDIDO COMPRA</t>
   </si>
   <si>
-    <t>ASSHA510646</t>
-  </si>
-  <si>
     <t>MSMU5779348</t>
   </si>
   <si>
@@ -415,9 +409,6 @@
     <t>29/10/2025</t>
   </si>
   <si>
-    <t>HTAO00015758</t>
-  </si>
-  <si>
     <t>MSBU5358793</t>
   </si>
   <si>
@@ -457,9 +448,6 @@
     <t>ZHANGZHOU WANHUI SANITARY WARE CO.,LTD</t>
   </si>
   <si>
-    <t>ASXMN503732</t>
-  </si>
-  <si>
     <t>MSMU5579458</t>
   </si>
   <si>
@@ -478,9 +466,6 @@
     <t>13/11/2025</t>
   </si>
   <si>
-    <t>ASXMN503730</t>
-  </si>
-  <si>
     <t>ZF1</t>
   </si>
   <si>
@@ -493,9 +478,6 @@
     <t>OLO-EPA/BINTER 35%</t>
   </si>
   <si>
-    <t>ASXMN503733</t>
-  </si>
-  <si>
     <t>MSMU5167532</t>
   </si>
   <si>
@@ -514,9 +496,6 @@
     <t>( 08/12/2025 08:12:19 - LEIDY ELIETH CHAVALA : «Se ha modificado el puerto de arribo. De: no tener puerto a: CALDERA, COSTA RICA» )</t>
   </si>
   <si>
-    <t>ASXMN503734</t>
-  </si>
-  <si>
     <t>ZF2</t>
   </si>
   <si>
@@ -532,9 +511,6 @@
     <t>JINNUO INDUSTRY (HK) CO., LIMITED</t>
   </si>
   <si>
-    <t>SZXD25168</t>
-  </si>
-  <si>
     <t>MEDU7373499</t>
   </si>
   <si>
@@ -553,9 +529,6 @@
     <t>( 10/12/2025 07:12:40 - LEIDY ELIETH CHAVALA : «Se ha modificado el puerto de embarque. De: no tener puerto a: SHEKOU, CHINA» )</t>
   </si>
   <si>
-    <t>SZXD25170</t>
-  </si>
-  <si>
     <t>ZF CA Oct 25 CNY #1</t>
   </si>
   <si>
@@ -616,12 +589,6 @@
     <t>OLO3</t>
   </si>
   <si>
-    <t>COSIARMA</t>
-  </si>
-  <si>
-    <t>SEALAND</t>
-  </si>
-  <si>
     <t>BILBAO, SPAIN</t>
   </si>
   <si>
@@ -641,13 +608,31 @@
   </si>
   <si>
     <t>BARRIOS, GUATEMALA</t>
+  </si>
+  <si>
+    <t>cmlbjeuyz0ohss66w2qlnjfck</t>
+  </si>
+  <si>
+    <t>Porth ID Raga</t>
+  </si>
+  <si>
+    <t>Porth ID Postman</t>
+  </si>
+  <si>
+    <t>cmlfkbdc70ldls66wl28wukpu</t>
+  </si>
+  <si>
+    <t>Naviera</t>
+  </si>
+  <si>
+    <t>Mediterranean Shipping</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -659,6 +644,12 @@
       <sz val="14"/>
       <color rgb="FF2E2E2E"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFCE9178"/>
+      <name val="Monaco"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -682,12 +673,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -992,8 +984,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BQ18"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:BQ33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="12" max="12" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20" bestFit="1" customWidth="1"/>
+    <col min="16" max="56" width="10.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:69" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -1204,7 +1202,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:69" ht="18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:69" ht="18" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>6701122</v>
       </c>
@@ -1308,13 +1306,13 @@
         <v>83</v>
       </c>
       <c r="AI2" s="4" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="AJ2" t="s">
         <v>73</v>
       </c>
       <c r="AK2" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AL2" t="s">
         <v>75</v>
@@ -1376,8 +1374,8 @@
       <c r="BE2" t="s">
         <v>78</v>
       </c>
-      <c r="BF2" s="4" t="s">
-        <v>193</v>
+      <c r="BF2" s="4" t="e">
+        <v>#N/A</v>
       </c>
       <c r="BG2" s="2">
         <v>45848</v>
@@ -1410,10 +1408,10 @@
         <v>71</v>
       </c>
       <c r="BQ2" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
-    <row r="3" spans="1:69" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:69" ht="18" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>6701206</v>
       </c>
@@ -1517,13 +1515,13 @@
         <v>92</v>
       </c>
       <c r="AI3" s="4" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="AJ3" t="s">
         <v>73</v>
       </c>
       <c r="AK3" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AM3" t="s">
         <v>71</v>
@@ -1582,8 +1580,8 @@
       <c r="BE3" t="s">
         <v>78</v>
       </c>
-      <c r="BF3" s="4" t="s">
-        <v>192</v>
+      <c r="BF3" s="4" t="e">
+        <v>#N/A</v>
       </c>
       <c r="BG3" s="2">
         <v>45698</v>
@@ -1616,10 +1614,10 @@
         <v>71</v>
       </c>
       <c r="BQ3" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
-    <row r="4" spans="1:69" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:69" ht="18" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>6701207</v>
       </c>
@@ -1723,13 +1721,13 @@
         <v>92</v>
       </c>
       <c r="AI4" s="4" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="AJ4" t="s">
         <v>73</v>
       </c>
       <c r="AK4" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AM4" t="s">
         <v>71</v>
@@ -1788,8 +1786,8 @@
       <c r="BE4" t="s">
         <v>78</v>
       </c>
-      <c r="BF4" s="4" t="s">
-        <v>192</v>
+      <c r="BF4" s="4" t="e">
+        <v>#N/A</v>
       </c>
       <c r="BG4" s="2">
         <v>45698</v>
@@ -1822,7 +1820,7 @@
         <v>71</v>
       </c>
       <c r="BQ4" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:69" ht="18" x14ac:dyDescent="0.2">
@@ -1859,14 +1857,11 @@
       <c r="K5">
         <v>2</v>
       </c>
-      <c r="L5" t="s">
-        <v>101</v>
-      </c>
       <c r="M5">
         <v>22</v>
       </c>
       <c r="N5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O5" t="s">
         <v>72</v>
@@ -1929,13 +1924,13 @@
         <v>74</v>
       </c>
       <c r="AI5" s="4" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="AJ5" t="s">
         <v>73</v>
       </c>
       <c r="AK5" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AL5" t="s">
         <v>75</v>
@@ -1962,13 +1957,13 @@
         <v>71</v>
       </c>
       <c r="AT5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AU5" s="3">
         <v>26948.92</v>
       </c>
       <c r="AV5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AW5" t="s">
         <v>76</v>
@@ -1995,10 +1990,10 @@
         <v>71</v>
       </c>
       <c r="BE5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="BF5" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="BG5" s="2">
         <v>45848</v>
@@ -2031,7 +2026,7 @@
         <v>71</v>
       </c>
       <c r="BQ5" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" spans="1:69" ht="18" x14ac:dyDescent="0.2">
@@ -2068,14 +2063,11 @@
       <c r="K6">
         <v>2</v>
       </c>
-      <c r="L6" t="s">
-        <v>106</v>
-      </c>
       <c r="M6">
         <v>22</v>
       </c>
       <c r="N6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="O6" t="s">
         <v>72</v>
@@ -2138,13 +2130,13 @@
         <v>74</v>
       </c>
       <c r="AI6" s="4" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="AJ6" t="s">
         <v>73</v>
       </c>
       <c r="AK6" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AL6" t="s">
         <v>75</v>
@@ -2171,13 +2163,13 @@
         <v>71</v>
       </c>
       <c r="AT6" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="AU6" s="3">
         <v>26985.119999999999</v>
       </c>
       <c r="AV6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="AW6" t="s">
         <v>76</v>
@@ -2204,10 +2196,10 @@
         <v>71</v>
       </c>
       <c r="BE6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="BF6" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="BG6" s="2">
         <v>45848</v>
@@ -2240,10 +2232,10 @@
         <v>71</v>
       </c>
       <c r="BQ6" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
-    <row r="7" spans="1:69" ht="18" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:69" ht="18" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6701353</v>
       </c>
@@ -2254,7 +2246,7 @@
         <v>270</v>
       </c>
       <c r="D7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E7">
         <v>88</v>
@@ -2278,13 +2270,13 @@
         <v>2</v>
       </c>
       <c r="L7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="M7">
         <v>23</v>
       </c>
       <c r="N7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="O7" t="s">
         <v>72</v>
@@ -2347,13 +2339,13 @@
         <v>74</v>
       </c>
       <c r="AI7" s="4" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="AJ7" t="s">
         <v>73</v>
       </c>
       <c r="AK7" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AL7" t="s">
         <v>75</v>
@@ -2365,7 +2357,7 @@
         <v>46009</v>
       </c>
       <c r="AO7" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="AP7" t="s">
         <v>71</v>
@@ -2380,13 +2372,13 @@
         <v>71</v>
       </c>
       <c r="AT7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="AU7" s="1">
         <v>17712</v>
       </c>
       <c r="AV7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="AW7" t="s">
         <v>76</v>
@@ -2398,7 +2390,7 @@
         <v>73</v>
       </c>
       <c r="AZ7" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="BA7" t="s">
         <v>76</v>
@@ -2415,8 +2407,8 @@
       <c r="BE7" t="s">
         <v>78</v>
       </c>
-      <c r="BF7" s="4" t="s">
-        <v>193</v>
+      <c r="BF7" s="4" t="e">
+        <v>#N/A</v>
       </c>
       <c r="BG7" s="2">
         <v>45848</v>
@@ -2449,10 +2441,10 @@
         <v>71</v>
       </c>
       <c r="BQ7" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
-    <row r="8" spans="1:69" ht="18" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:69" ht="18" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>6701683</v>
       </c>
@@ -2463,7 +2455,7 @@
         <v>380</v>
       </c>
       <c r="D8" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E8">
         <v>85</v>
@@ -2487,13 +2479,13 @@
         <v>2</v>
       </c>
       <c r="L8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="M8">
         <v>23</v>
       </c>
       <c r="N8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="O8" t="s">
         <v>72</v>
@@ -2556,13 +2548,13 @@
         <v>74</v>
       </c>
       <c r="AI8" s="4" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="AJ8" t="s">
         <v>73</v>
       </c>
       <c r="AK8" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AL8" t="s">
         <v>75</v>
@@ -2574,7 +2566,7 @@
         <v>46001</v>
       </c>
       <c r="AO8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="AP8" t="s">
         <v>71</v>
@@ -2589,13 +2581,13 @@
         <v>71</v>
       </c>
       <c r="AT8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="AU8" s="3">
         <v>20570.05</v>
       </c>
       <c r="AV8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="AW8" t="s">
         <v>76</v>
@@ -2607,7 +2599,7 @@
         <v>73</v>
       </c>
       <c r="AZ8" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="BA8" t="s">
         <v>76</v>
@@ -2624,11 +2616,11 @@
       <c r="BE8" t="s">
         <v>78</v>
       </c>
-      <c r="BF8" s="4" t="s">
-        <v>193</v>
+      <c r="BF8" s="4" t="e">
+        <v>#N/A</v>
       </c>
       <c r="BG8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="BH8">
         <v>14</v>
@@ -2658,7 +2650,7 @@
         <v>71</v>
       </c>
       <c r="BQ8" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9" spans="1:69" ht="18" x14ac:dyDescent="0.2">
@@ -2672,7 +2664,7 @@
         <v>380</v>
       </c>
       <c r="D9" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E9">
         <v>85</v>
@@ -2695,14 +2687,11 @@
       <c r="K9">
         <v>2</v>
       </c>
-      <c r="L9" t="s">
-        <v>125</v>
-      </c>
       <c r="M9">
         <v>23</v>
       </c>
       <c r="N9" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="O9" t="s">
         <v>72</v>
@@ -2765,13 +2754,13 @@
         <v>74</v>
       </c>
       <c r="AI9" s="4" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="AJ9" t="s">
         <v>73</v>
       </c>
       <c r="AK9" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AL9" t="s">
         <v>75</v>
@@ -2783,7 +2772,7 @@
         <v>46001</v>
       </c>
       <c r="AO9" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="AP9" t="s">
         <v>71</v>
@@ -2798,13 +2787,13 @@
         <v>71</v>
       </c>
       <c r="AT9" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="AU9" s="3">
         <v>20570.05</v>
       </c>
       <c r="AV9" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="AW9" t="s">
         <v>76</v>
@@ -2816,7 +2805,7 @@
         <v>73</v>
       </c>
       <c r="AZ9" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="BA9" t="s">
         <v>76</v>
@@ -2834,10 +2823,10 @@
         <v>78</v>
       </c>
       <c r="BF9" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="BG9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="BH9">
         <v>14</v>
@@ -2867,10 +2856,10 @@
         <v>71</v>
       </c>
       <c r="BQ9" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
-    <row r="10" spans="1:69" ht="18" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:69" ht="18" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>6701758</v>
       </c>
@@ -2881,7 +2870,7 @@
         <v>903</v>
       </c>
       <c r="D10" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E10">
         <v>85</v>
@@ -2905,13 +2894,13 @@
         <v>2</v>
       </c>
       <c r="L10" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="M10">
         <v>23</v>
       </c>
       <c r="N10" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="O10" t="s">
         <v>72</v>
@@ -2974,13 +2963,13 @@
         <v>92</v>
       </c>
       <c r="AI10" s="4" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="AJ10" t="s">
         <v>73</v>
       </c>
       <c r="AK10" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AM10" t="s">
         <v>71</v>
@@ -2989,7 +2978,7 @@
         <v>71</v>
       </c>
       <c r="AO10" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="AP10" t="s">
         <v>71</v>
@@ -3004,13 +2993,13 @@
         <v>71</v>
       </c>
       <c r="AT10" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="AU10" s="3">
         <v>29145.119999999999</v>
       </c>
       <c r="AV10" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="AW10" t="s">
         <v>76</v>
@@ -3022,7 +3011,7 @@
         <v>76</v>
       </c>
       <c r="AZ10" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="BA10" t="s">
         <v>73</v>
@@ -3039,8 +3028,8 @@
       <c r="BE10" t="s">
         <v>78</v>
       </c>
-      <c r="BF10" s="4" t="s">
-        <v>193</v>
+      <c r="BF10" s="4" t="e">
+        <v>#N/A</v>
       </c>
       <c r="BG10" s="2">
         <v>45972</v>
@@ -3073,7 +3062,7 @@
         <v>71</v>
       </c>
       <c r="BQ10" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11" spans="1:69" ht="18" x14ac:dyDescent="0.2">
@@ -3087,7 +3076,7 @@
         <v>905</v>
       </c>
       <c r="D11" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="E11">
         <v>89</v>
@@ -3110,14 +3099,11 @@
       <c r="K11">
         <v>2</v>
       </c>
-      <c r="L11" t="s">
-        <v>139</v>
-      </c>
       <c r="M11">
         <v>23</v>
       </c>
       <c r="N11" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="O11" t="s">
         <v>72</v>
@@ -3180,13 +3166,13 @@
         <v>74</v>
       </c>
       <c r="AI11" s="4" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="AJ11" t="s">
         <v>73</v>
       </c>
       <c r="AK11" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AL11" t="s">
         <v>75</v>
@@ -3198,7 +3184,7 @@
         <v>45999</v>
       </c>
       <c r="AO11" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="AP11" t="s">
         <v>71</v>
@@ -3213,19 +3199,19 @@
         <v>71</v>
       </c>
       <c r="AT11" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="AU11" s="1">
         <v>13860</v>
       </c>
       <c r="AV11" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="AW11" t="s">
         <v>76</v>
       </c>
       <c r="AX11" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="AY11" t="s">
         <v>76</v>
@@ -3249,10 +3235,10 @@
         <v>78</v>
       </c>
       <c r="BF11" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="BG11" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="BH11">
         <v>14</v>
@@ -3282,7 +3268,7 @@
         <v>71</v>
       </c>
       <c r="BQ11" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12" spans="1:69" ht="18" x14ac:dyDescent="0.2">
@@ -3296,7 +3282,7 @@
         <v>905</v>
       </c>
       <c r="D12" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="E12">
         <v>89</v>
@@ -3319,14 +3305,11 @@
       <c r="K12">
         <v>2</v>
       </c>
-      <c r="L12" t="s">
-        <v>146</v>
-      </c>
       <c r="M12">
         <v>23</v>
       </c>
       <c r="N12" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="O12" t="s">
         <v>72</v>
@@ -3389,13 +3372,13 @@
         <v>92</v>
       </c>
       <c r="AI12" s="4" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="AJ12" t="s">
         <v>73</v>
       </c>
       <c r="AK12" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AM12" t="s">
         <v>71</v>
@@ -3404,7 +3387,7 @@
         <v>71</v>
       </c>
       <c r="AO12" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="AP12" t="s">
         <v>71</v>
@@ -3419,19 +3402,19 @@
         <v>71</v>
       </c>
       <c r="AT12" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="AU12" s="1">
         <v>5841</v>
       </c>
       <c r="AV12" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="AW12" t="s">
         <v>76</v>
       </c>
       <c r="AX12" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="AY12" t="s">
         <v>76</v>
@@ -3455,10 +3438,10 @@
         <v>78</v>
       </c>
       <c r="BF12" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="BG12" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="BH12">
         <v>14</v>
@@ -3488,7 +3471,7 @@
         <v>71</v>
       </c>
       <c r="BQ12" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13" spans="1:69" ht="18" x14ac:dyDescent="0.2">
@@ -3502,7 +3485,7 @@
         <v>905</v>
       </c>
       <c r="D13" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="E13">
         <v>89</v>
@@ -3525,14 +3508,11 @@
       <c r="K13">
         <v>2</v>
       </c>
-      <c r="L13" t="s">
-        <v>151</v>
-      </c>
       <c r="M13">
         <v>23</v>
       </c>
       <c r="N13" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="O13" t="s">
         <v>72</v>
@@ -3595,13 +3575,13 @@
         <v>74</v>
       </c>
       <c r="AI13" s="4" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="AJ13" t="s">
         <v>73</v>
       </c>
       <c r="AK13" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AL13" t="s">
         <v>75</v>
@@ -3613,7 +3593,7 @@
         <v>45999</v>
       </c>
       <c r="AO13" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="AP13" t="s">
         <v>71</v>
@@ -3628,25 +3608,25 @@
         <v>71</v>
       </c>
       <c r="AT13" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="AU13" s="1">
         <v>2720</v>
       </c>
       <c r="AV13" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="AW13" t="s">
         <v>76</v>
       </c>
       <c r="AX13" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="AY13" t="s">
         <v>76</v>
       </c>
       <c r="AZ13" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="BA13" t="s">
         <v>76</v>
@@ -3664,10 +3644,10 @@
         <v>78</v>
       </c>
       <c r="BF13" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="BG13" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="BH13">
         <v>14</v>
@@ -3697,7 +3677,7 @@
         <v>71</v>
       </c>
       <c r="BQ13" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="14" spans="1:69" ht="18" x14ac:dyDescent="0.2">
@@ -3711,7 +3691,7 @@
         <v>905</v>
       </c>
       <c r="D14" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="E14">
         <v>89</v>
@@ -3734,14 +3714,11 @@
       <c r="K14">
         <v>2</v>
       </c>
-      <c r="L14" t="s">
-        <v>158</v>
-      </c>
       <c r="M14">
         <v>23</v>
       </c>
       <c r="N14" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="O14" t="s">
         <v>72</v>
@@ -3804,13 +3781,13 @@
         <v>92</v>
       </c>
       <c r="AI14" s="4" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="AJ14" t="s">
         <v>73</v>
       </c>
       <c r="AK14" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AM14" t="s">
         <v>71</v>
@@ -3819,7 +3796,7 @@
         <v>71</v>
       </c>
       <c r="AO14" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="AP14" t="s">
         <v>71</v>
@@ -3834,19 +3811,19 @@
         <v>71</v>
       </c>
       <c r="AT14" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="AU14" s="1">
         <v>18305</v>
       </c>
       <c r="AV14" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="AW14" t="s">
         <v>76</v>
       </c>
       <c r="AX14" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="AY14" t="s">
         <v>76</v>
@@ -3870,10 +3847,10 @@
         <v>78</v>
       </c>
       <c r="BF14" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="BG14" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="BH14">
         <v>14</v>
@@ -3903,7 +3880,7 @@
         <v>71</v>
       </c>
       <c r="BQ14" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="15" spans="1:69" ht="18" x14ac:dyDescent="0.2">
@@ -3917,7 +3894,7 @@
         <v>913</v>
       </c>
       <c r="D15" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="E15">
         <v>85</v>
@@ -3940,14 +3917,11 @@
       <c r="K15">
         <v>2</v>
       </c>
-      <c r="L15" t="s">
-        <v>164</v>
-      </c>
       <c r="M15">
         <v>23</v>
       </c>
       <c r="N15" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="O15" t="s">
         <v>72</v>
@@ -4010,13 +3984,13 @@
         <v>74</v>
       </c>
       <c r="AI15" s="4" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="AJ15" t="s">
         <v>73</v>
       </c>
       <c r="AK15" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AL15" t="s">
         <v>75</v>
@@ -4028,7 +4002,7 @@
         <v>46008</v>
       </c>
       <c r="AO15" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="AP15" t="s">
         <v>71</v>
@@ -4043,25 +4017,25 @@
         <v>71</v>
       </c>
       <c r="AT15" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="AU15" s="1">
         <v>13090</v>
       </c>
       <c r="AV15" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="AW15" t="s">
         <v>76</v>
       </c>
       <c r="AX15" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="AY15" t="s">
         <v>76</v>
       </c>
       <c r="AZ15" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="BA15" t="s">
         <v>76</v>
@@ -4079,7 +4053,7 @@
         <v>78</v>
       </c>
       <c r="BF15" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="BG15" s="2">
         <v>45700</v>
@@ -4112,7 +4086,7 @@
         <v>71</v>
       </c>
       <c r="BQ15" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16" spans="1:69" ht="18" x14ac:dyDescent="0.2">
@@ -4126,7 +4100,7 @@
         <v>913</v>
       </c>
       <c r="D16" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="E16">
         <v>85</v>
@@ -4149,14 +4123,11 @@
       <c r="K16">
         <v>2</v>
       </c>
-      <c r="L16" t="s">
-        <v>171</v>
-      </c>
       <c r="M16">
         <v>23</v>
       </c>
       <c r="N16" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="O16" t="s">
         <v>72</v>
@@ -4219,13 +4190,13 @@
         <v>92</v>
       </c>
       <c r="AI16" s="4" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="AJ16" t="s">
         <v>73</v>
       </c>
       <c r="AK16" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AM16" t="s">
         <v>71</v>
@@ -4234,7 +4205,7 @@
         <v>71</v>
       </c>
       <c r="AO16" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="AP16" t="s">
         <v>71</v>
@@ -4249,25 +4220,25 @@
         <v>71</v>
       </c>
       <c r="AT16" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="AU16" s="1">
         <v>5950</v>
       </c>
       <c r="AV16" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="AW16" t="s">
         <v>76</v>
       </c>
       <c r="AX16" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="AY16" t="s">
         <v>76</v>
       </c>
       <c r="AZ16" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="BA16" t="s">
         <v>76</v>
@@ -4285,7 +4256,7 @@
         <v>78</v>
       </c>
       <c r="BF16" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="BG16" s="2">
         <v>45700</v>
@@ -4318,10 +4289,10 @@
         <v>71</v>
       </c>
       <c r="BQ16" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
-    <row r="17" spans="1:69" ht="18" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:69" ht="18" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>6702106</v>
       </c>
@@ -4332,7 +4303,7 @@
         <v>494</v>
       </c>
       <c r="D17" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="E17">
         <v>83</v>
@@ -4356,13 +4327,13 @@
         <v>2</v>
       </c>
       <c r="L17" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="M17">
         <v>21</v>
       </c>
       <c r="N17" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="O17" t="s">
         <v>72</v>
@@ -4425,13 +4396,13 @@
         <v>74</v>
       </c>
       <c r="AI17" s="4" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="AJ17" t="s">
         <v>73</v>
       </c>
       <c r="AK17" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AL17" t="s">
         <v>75</v>
@@ -4443,7 +4414,7 @@
         <v>46055</v>
       </c>
       <c r="AO17" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="AP17" t="s">
         <v>71</v>
@@ -4458,19 +4429,19 @@
         <v>71</v>
       </c>
       <c r="AT17" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="AU17" s="3">
         <v>22673.74</v>
       </c>
       <c r="AV17" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="AW17" t="s">
         <v>76</v>
       </c>
       <c r="AX17" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="AY17" t="s">
         <v>73</v>
@@ -4493,8 +4464,8 @@
       <c r="BE17" t="s">
         <v>78</v>
       </c>
-      <c r="BF17" s="4" t="s">
-        <v>192</v>
+      <c r="BF17" s="4" t="e">
+        <v>#N/A</v>
       </c>
       <c r="BG17" s="2">
         <v>45819</v>
@@ -4527,10 +4498,10 @@
         <v>71</v>
       </c>
       <c r="BQ17" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
-    <row r="18" spans="1:69" ht="18" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:69" ht="18" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>6702107</v>
       </c>
@@ -4541,7 +4512,7 @@
         <v>494</v>
       </c>
       <c r="D18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="E18">
         <v>83</v>
@@ -4565,13 +4536,13 @@
         <v>2</v>
       </c>
       <c r="L18" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="M18">
         <v>25</v>
       </c>
       <c r="N18" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="O18" t="s">
         <v>72</v>
@@ -4634,13 +4605,13 @@
         <v>92</v>
       </c>
       <c r="AI18" s="4" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="AJ18" t="s">
         <v>73</v>
       </c>
       <c r="AK18" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="AM18" t="s">
         <v>71</v>
@@ -4649,7 +4620,7 @@
         <v>71</v>
       </c>
       <c r="AO18" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="AP18" t="s">
         <v>71</v>
@@ -4664,25 +4635,25 @@
         <v>71</v>
       </c>
       <c r="AT18" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="AU18" s="3">
         <v>58880.98</v>
       </c>
       <c r="AV18" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="AW18" t="s">
         <v>76</v>
       </c>
       <c r="AX18" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="AY18" t="s">
         <v>76</v>
       </c>
       <c r="AZ18" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="BA18" t="s">
         <v>76</v>
@@ -4697,10 +4668,10 @@
         <v>71</v>
       </c>
       <c r="BE18" t="s">
-        <v>190</v>
-      </c>
-      <c r="BF18" s="4" t="s">
-        <v>192</v>
+        <v>181</v>
+      </c>
+      <c r="BF18" s="4" t="e">
+        <v>#N/A</v>
       </c>
       <c r="BG18" s="2">
         <v>45819</v>
@@ -4733,11 +4704,143 @@
         <v>71</v>
       </c>
       <c r="BQ18" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="22" spans="1:69" x14ac:dyDescent="0.2">
+      <c r="K22" t="s">
         <v>191</v>
+      </c>
+      <c r="L22" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="23" spans="1:69" ht="16" x14ac:dyDescent="0.2">
+      <c r="K23" t="s">
+        <v>192</v>
+      </c>
+      <c r="L23" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="24" spans="1:69" x14ac:dyDescent="0.2">
+      <c r="BF24" t="s">
+        <v>0</v>
+      </c>
+      <c r="BG24" t="s">
+        <v>194</v>
+      </c>
+      <c r="BH24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:69" x14ac:dyDescent="0.2">
+      <c r="BF25">
+        <v>6701296</v>
+      </c>
+      <c r="BG25" t="s">
+        <v>195</v>
+      </c>
+      <c r="BH25" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="26" spans="1:69" x14ac:dyDescent="0.2">
+      <c r="BF26">
+        <v>6701297</v>
+      </c>
+      <c r="BG26" t="s">
+        <v>195</v>
+      </c>
+      <c r="BH26" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="27" spans="1:69" x14ac:dyDescent="0.2">
+      <c r="BF27">
+        <v>6701684</v>
+      </c>
+      <c r="BG27" t="s">
+        <v>195</v>
+      </c>
+      <c r="BH27" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="28" spans="1:69" x14ac:dyDescent="0.2">
+      <c r="BF28">
+        <v>6701769</v>
+      </c>
+      <c r="BG28" t="s">
+        <v>195</v>
+      </c>
+      <c r="BH28" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="29" spans="1:69" x14ac:dyDescent="0.2">
+      <c r="BF29">
+        <v>6701770</v>
+      </c>
+      <c r="BG29" t="s">
+        <v>195</v>
+      </c>
+      <c r="BH29" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="30" spans="1:69" x14ac:dyDescent="0.2">
+      <c r="BF30">
+        <v>6701771</v>
+      </c>
+      <c r="BG30" t="s">
+        <v>195</v>
+      </c>
+      <c r="BH30" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="31" spans="1:69" x14ac:dyDescent="0.2">
+      <c r="BF31">
+        <v>6701772</v>
+      </c>
+      <c r="BG31" t="s">
+        <v>195</v>
+      </c>
+      <c r="BH31" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="32" spans="1:69" x14ac:dyDescent="0.2">
+      <c r="BF32">
+        <v>6702103</v>
+      </c>
+      <c r="BG32" t="s">
+        <v>195</v>
+      </c>
+      <c r="BH32" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="33" spans="58:60" x14ac:dyDescent="0.2">
+      <c r="BF33">
+        <v>6702104</v>
+      </c>
+      <c r="BG33" t="s">
+        <v>195</v>
+      </c>
+      <c r="BH33" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BQ18" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:BQ18" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="57">
+      <filters>
+        <filter val="Mediterranean Shipping"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>